<commit_message>
Add Image Mapper so artist images with any file name can be installed
Kitefall > Art > Image Mapper matches images to the 278 slots of the image
list (auto-match by name, by row number, from CSV, or by drag and drop),
renames and moves them into Resources/KitefallArt, applies mobile import
settings and sets the app icon. The game uses installed images for kite
skins, shop and wardrobe cards, portraits, menu backgrounds, splash/logo and
HUD icons, and falls back to the generated look when an image is missing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kft94361aqxz3Q9WMshigR
</commit_message>
<xml_diff>
--- a/docs/Kitefall_Image_Assets.xlsx
+++ b/docs/Kitefall_Image_Assets.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image List" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$L$279</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$M$279</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -690,13 +690,25 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Different file names?</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>No problem. In Unity open Kitefall &gt; Art &gt; Image Mapper. Drag each image onto its slot, or press Auto-match. Or type your own file name in the last column of 'Image List', save this sheet as CSV and press 'Import CSV' in the mapper. Files named only with the # number (e.g. 45.png) can be matched with 'Match by # number'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Licence check</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Use an AI tool whose terms allow commercial use, and keep the prompt + date for every final image (record it in the 'Status / notes' column).</t>
         </is>
@@ -1325,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L279"/>
+  <dimension ref="A1:M279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1352,7 @@
     <col width="50" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1403,6 +1416,11 @@
           <t>Status / notes</t>
         </is>
       </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Your file name (fill if different)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="120" customHeight="1">
       <c r="A2" s="7" t="n">
@@ -1459,6 +1477,7 @@
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="inlineStr"/>
     </row>
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="9" t="n">
@@ -1515,6 +1534,7 @@
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr"/>
     </row>
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="7" t="n">
@@ -1571,6 +1591,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr"/>
     </row>
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="9" t="n">
@@ -1627,6 +1648,7 @@
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr"/>
     </row>
     <row r="6" ht="120" customHeight="1">
       <c r="A6" s="7" t="n">
@@ -1683,6 +1705,7 @@
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr"/>
+      <c r="M6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="120" customHeight="1">
       <c r="A7" s="9" t="n">
@@ -1739,6 +1762,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="inlineStr"/>
+      <c r="M7" s="9" t="inlineStr"/>
     </row>
     <row r="8" ht="120" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -1795,6 +1819,7 @@
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="120" customHeight="1">
       <c r="A9" s="9" t="n">
@@ -1851,6 +1876,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr"/>
+      <c r="M9" s="9" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -1907,6 +1933,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr"/>
+      <c r="M10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="9" t="n">
@@ -1963,6 +1990,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr"/>
+      <c r="M11" s="9" t="inlineStr"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -2019,6 +2047,7 @@
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="9" t="n">
@@ -2075,6 +2104,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr"/>
     </row>
     <row r="14" ht="120" customHeight="1">
       <c r="A14" s="7" t="n">
@@ -2131,6 +2161,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr"/>
+      <c r="M14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="120" customHeight="1">
       <c r="A15" s="9" t="n">
@@ -2187,6 +2218,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="inlineStr"/>
+      <c r="M15" s="9" t="inlineStr"/>
     </row>
     <row r="16" ht="120" customHeight="1">
       <c r="A16" s="7" t="n">
@@ -2243,6 +2275,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="120" customHeight="1">
       <c r="A17" s="9" t="n">
@@ -2299,6 +2332,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="inlineStr"/>
+      <c r="M17" s="9" t="inlineStr"/>
     </row>
     <row r="18" ht="120" customHeight="1">
       <c r="A18" s="7" t="n">
@@ -2355,6 +2389,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr"/>
+      <c r="M18" s="7" t="inlineStr"/>
     </row>
     <row r="19" ht="120" customHeight="1">
       <c r="A19" s="9" t="n">
@@ -2411,6 +2446,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="inlineStr"/>
+      <c r="M19" s="9" t="inlineStr"/>
     </row>
     <row r="20" ht="120" customHeight="1">
       <c r="A20" s="7" t="n">
@@ -2467,6 +2503,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr"/>
+      <c r="M20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="9" t="n">
@@ -2523,6 +2560,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="inlineStr"/>
+      <c r="M21" s="9" t="inlineStr"/>
     </row>
     <row r="22" ht="120" customHeight="1">
       <c r="A22" s="7" t="n">
@@ -2579,6 +2617,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr"/>
+      <c r="M22" s="7" t="inlineStr"/>
     </row>
     <row r="23" ht="120" customHeight="1">
       <c r="A23" s="9" t="n">
@@ -2635,6 +2674,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr"/>
+      <c r="M23" s="9" t="inlineStr"/>
     </row>
     <row r="24" ht="120" customHeight="1">
       <c r="A24" s="7" t="n">
@@ -2691,6 +2731,7 @@
         </is>
       </c>
       <c r="L24" s="7" t="inlineStr"/>
+      <c r="M24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="120" customHeight="1">
       <c r="A25" s="9" t="n">
@@ -2747,6 +2788,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="inlineStr"/>
+      <c r="M25" s="9" t="inlineStr"/>
     </row>
     <row r="26" ht="120" customHeight="1">
       <c r="A26" s="7" t="n">
@@ -2803,6 +2845,7 @@
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr"/>
+      <c r="M26" s="7" t="inlineStr"/>
     </row>
     <row r="27" ht="120" customHeight="1">
       <c r="A27" s="9" t="n">
@@ -2859,6 +2902,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="inlineStr"/>
+      <c r="M27" s="9" t="inlineStr"/>
     </row>
     <row r="28" ht="120" customHeight="1">
       <c r="A28" s="7" t="n">
@@ -2915,6 +2959,7 @@
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr"/>
+      <c r="M28" s="7" t="inlineStr"/>
     </row>
     <row r="29" ht="120" customHeight="1">
       <c r="A29" s="9" t="n">
@@ -2971,6 +3016,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="inlineStr"/>
+      <c r="M29" s="9" t="inlineStr"/>
     </row>
     <row r="30" ht="120" customHeight="1">
       <c r="A30" s="7" t="n">
@@ -3027,6 +3073,7 @@
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr"/>
+      <c r="M30" s="7" t="inlineStr"/>
     </row>
     <row r="31" ht="120" customHeight="1">
       <c r="A31" s="9" t="n">
@@ -3083,6 +3130,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="inlineStr"/>
+      <c r="M31" s="9" t="inlineStr"/>
     </row>
     <row r="32" ht="120" customHeight="1">
       <c r="A32" s="7" t="n">
@@ -3139,6 +3187,7 @@
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr"/>
+      <c r="M32" s="7" t="inlineStr"/>
     </row>
     <row r="33" ht="120" customHeight="1">
       <c r="A33" s="9" t="n">
@@ -3195,6 +3244,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="inlineStr"/>
+      <c r="M33" s="9" t="inlineStr"/>
     </row>
     <row r="34" ht="120" customHeight="1">
       <c r="A34" s="7" t="n">
@@ -3251,6 +3301,7 @@
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr"/>
+      <c r="M34" s="7" t="inlineStr"/>
     </row>
     <row r="35" ht="120" customHeight="1">
       <c r="A35" s="9" t="n">
@@ -3307,6 +3358,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="inlineStr"/>
+      <c r="M35" s="9" t="inlineStr"/>
     </row>
     <row r="36" ht="120" customHeight="1">
       <c r="A36" s="7" t="n">
@@ -3363,6 +3415,7 @@
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr"/>
+      <c r="M36" s="7" t="inlineStr"/>
     </row>
     <row r="37" ht="120" customHeight="1">
       <c r="A37" s="9" t="n">
@@ -3419,6 +3472,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="inlineStr"/>
+      <c r="M37" s="9" t="inlineStr"/>
     </row>
     <row r="38" ht="120" customHeight="1">
       <c r="A38" s="7" t="n">
@@ -3475,6 +3529,7 @@
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr"/>
+      <c r="M38" s="7" t="inlineStr"/>
     </row>
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="9" t="n">
@@ -3531,6 +3586,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="inlineStr"/>
+      <c r="M39" s="9" t="inlineStr"/>
     </row>
     <row r="40" ht="120" customHeight="1">
       <c r="A40" s="7" t="n">
@@ -3587,6 +3643,7 @@
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr"/>
+      <c r="M40" s="7" t="inlineStr"/>
     </row>
     <row r="41" ht="120" customHeight="1">
       <c r="A41" s="9" t="n">
@@ -3643,6 +3700,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="inlineStr"/>
+      <c r="M41" s="9" t="inlineStr"/>
     </row>
     <row r="42" ht="120" customHeight="1">
       <c r="A42" s="7" t="n">
@@ -3699,6 +3757,7 @@
         </is>
       </c>
       <c r="L42" s="7" t="inlineStr"/>
+      <c r="M42" s="7" t="inlineStr"/>
     </row>
     <row r="43" ht="120" customHeight="1">
       <c r="A43" s="9" t="n">
@@ -3755,6 +3814,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="inlineStr"/>
+      <c r="M43" s="9" t="inlineStr"/>
     </row>
     <row r="44" ht="120" customHeight="1">
       <c r="A44" s="7" t="n">
@@ -3811,6 +3871,7 @@
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr"/>
+      <c r="M44" s="7" t="inlineStr"/>
     </row>
     <row r="45" ht="120" customHeight="1">
       <c r="A45" s="9" t="n">
@@ -3867,6 +3928,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="inlineStr"/>
+      <c r="M45" s="9" t="inlineStr"/>
     </row>
     <row r="46" ht="120" customHeight="1">
       <c r="A46" s="7" t="n">
@@ -3923,6 +3985,7 @@
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr"/>
+      <c r="M46" s="7" t="inlineStr"/>
     </row>
     <row r="47" ht="120" customHeight="1">
       <c r="A47" s="9" t="n">
@@ -3979,6 +4042,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="inlineStr"/>
+      <c r="M47" s="9" t="inlineStr"/>
     </row>
     <row r="48" ht="120" customHeight="1">
       <c r="A48" s="7" t="n">
@@ -4035,6 +4099,7 @@
         </is>
       </c>
       <c r="L48" s="7" t="inlineStr"/>
+      <c r="M48" s="7" t="inlineStr"/>
     </row>
     <row r="49" ht="120" customHeight="1">
       <c r="A49" s="9" t="n">
@@ -4091,6 +4156,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="inlineStr"/>
+      <c r="M49" s="9" t="inlineStr"/>
     </row>
     <row r="50" ht="120" customHeight="1">
       <c r="A50" s="7" t="n">
@@ -4147,6 +4213,7 @@
         </is>
       </c>
       <c r="L50" s="7" t="inlineStr"/>
+      <c r="M50" s="7" t="inlineStr"/>
     </row>
     <row r="51" ht="120" customHeight="1">
       <c r="A51" s="9" t="n">
@@ -4203,6 +4270,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="inlineStr"/>
+      <c r="M51" s="9" t="inlineStr"/>
     </row>
     <row r="52" ht="120" customHeight="1">
       <c r="A52" s="7" t="n">
@@ -4259,6 +4327,7 @@
         </is>
       </c>
       <c r="L52" s="7" t="inlineStr"/>
+      <c r="M52" s="7" t="inlineStr"/>
     </row>
     <row r="53" ht="120" customHeight="1">
       <c r="A53" s="9" t="n">
@@ -4315,6 +4384,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="inlineStr"/>
+      <c r="M53" s="9" t="inlineStr"/>
     </row>
     <row r="54" ht="120" customHeight="1">
       <c r="A54" s="7" t="n">
@@ -4371,6 +4441,7 @@
         </is>
       </c>
       <c r="L54" s="7" t="inlineStr"/>
+      <c r="M54" s="7" t="inlineStr"/>
     </row>
     <row r="55" ht="120" customHeight="1">
       <c r="A55" s="9" t="n">
@@ -4427,6 +4498,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="inlineStr"/>
+      <c r="M55" s="9" t="inlineStr"/>
     </row>
     <row r="56" ht="120" customHeight="1">
       <c r="A56" s="7" t="n">
@@ -4483,6 +4555,7 @@
         </is>
       </c>
       <c r="L56" s="7" t="inlineStr"/>
+      <c r="M56" s="7" t="inlineStr"/>
     </row>
     <row r="57" ht="120" customHeight="1">
       <c r="A57" s="9" t="n">
@@ -4539,6 +4612,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="inlineStr"/>
+      <c r="M57" s="9" t="inlineStr"/>
     </row>
     <row r="58" ht="120" customHeight="1">
       <c r="A58" s="7" t="n">
@@ -4595,6 +4669,7 @@
         </is>
       </c>
       <c r="L58" s="7" t="inlineStr"/>
+      <c r="M58" s="7" t="inlineStr"/>
     </row>
     <row r="59" ht="120" customHeight="1">
       <c r="A59" s="9" t="n">
@@ -4651,6 +4726,7 @@
         </is>
       </c>
       <c r="L59" s="9" t="inlineStr"/>
+      <c r="M59" s="9" t="inlineStr"/>
     </row>
     <row r="60" ht="120" customHeight="1">
       <c r="A60" s="7" t="n">
@@ -4707,6 +4783,7 @@
         </is>
       </c>
       <c r="L60" s="7" t="inlineStr"/>
+      <c r="M60" s="7" t="inlineStr"/>
     </row>
     <row r="61" ht="120" customHeight="1">
       <c r="A61" s="9" t="n">
@@ -4763,6 +4840,7 @@
         </is>
       </c>
       <c r="L61" s="9" t="inlineStr"/>
+      <c r="M61" s="9" t="inlineStr"/>
     </row>
     <row r="62" ht="120" customHeight="1">
       <c r="A62" s="7" t="n">
@@ -4819,6 +4897,7 @@
         </is>
       </c>
       <c r="L62" s="7" t="inlineStr"/>
+      <c r="M62" s="7" t="inlineStr"/>
     </row>
     <row r="63" ht="120" customHeight="1">
       <c r="A63" s="9" t="n">
@@ -4875,6 +4954,7 @@
         </is>
       </c>
       <c r="L63" s="9" t="inlineStr"/>
+      <c r="M63" s="9" t="inlineStr"/>
     </row>
     <row r="64" ht="120" customHeight="1">
       <c r="A64" s="7" t="n">
@@ -4931,6 +5011,7 @@
         </is>
       </c>
       <c r="L64" s="7" t="inlineStr"/>
+      <c r="M64" s="7" t="inlineStr"/>
     </row>
     <row r="65" ht="120" customHeight="1">
       <c r="A65" s="9" t="n">
@@ -4987,6 +5068,7 @@
         </is>
       </c>
       <c r="L65" s="9" t="inlineStr"/>
+      <c r="M65" s="9" t="inlineStr"/>
     </row>
     <row r="66" ht="120" customHeight="1">
       <c r="A66" s="7" t="n">
@@ -5043,6 +5125,7 @@
         </is>
       </c>
       <c r="L66" s="7" t="inlineStr"/>
+      <c r="M66" s="7" t="inlineStr"/>
     </row>
     <row r="67" ht="120" customHeight="1">
       <c r="A67" s="9" t="n">
@@ -5099,6 +5182,7 @@
         </is>
       </c>
       <c r="L67" s="9" t="inlineStr"/>
+      <c r="M67" s="9" t="inlineStr"/>
     </row>
     <row r="68" ht="120" customHeight="1">
       <c r="A68" s="7" t="n">
@@ -5155,6 +5239,7 @@
         </is>
       </c>
       <c r="L68" s="7" t="inlineStr"/>
+      <c r="M68" s="7" t="inlineStr"/>
     </row>
     <row r="69" ht="120" customHeight="1">
       <c r="A69" s="9" t="n">
@@ -5211,6 +5296,7 @@
         </is>
       </c>
       <c r="L69" s="9" t="inlineStr"/>
+      <c r="M69" s="9" t="inlineStr"/>
     </row>
     <row r="70" ht="120" customHeight="1">
       <c r="A70" s="7" t="n">
@@ -5267,6 +5353,7 @@
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr"/>
+      <c r="M70" s="7" t="inlineStr"/>
     </row>
     <row r="71" ht="120" customHeight="1">
       <c r="A71" s="9" t="n">
@@ -5323,6 +5410,7 @@
         </is>
       </c>
       <c r="L71" s="9" t="inlineStr"/>
+      <c r="M71" s="9" t="inlineStr"/>
     </row>
     <row r="72" ht="120" customHeight="1">
       <c r="A72" s="7" t="n">
@@ -5379,6 +5467,7 @@
         </is>
       </c>
       <c r="L72" s="7" t="inlineStr"/>
+      <c r="M72" s="7" t="inlineStr"/>
     </row>
     <row r="73" ht="120" customHeight="1">
       <c r="A73" s="9" t="n">
@@ -5435,6 +5524,7 @@
         </is>
       </c>
       <c r="L73" s="9" t="inlineStr"/>
+      <c r="M73" s="9" t="inlineStr"/>
     </row>
     <row r="74" ht="120" customHeight="1">
       <c r="A74" s="7" t="n">
@@ -5491,6 +5581,7 @@
         </is>
       </c>
       <c r="L74" s="7" t="inlineStr"/>
+      <c r="M74" s="7" t="inlineStr"/>
     </row>
     <row r="75" ht="120" customHeight="1">
       <c r="A75" s="9" t="n">
@@ -5547,6 +5638,7 @@
         </is>
       </c>
       <c r="L75" s="9" t="inlineStr"/>
+      <c r="M75" s="9" t="inlineStr"/>
     </row>
     <row r="76" ht="120" customHeight="1">
       <c r="A76" s="7" t="n">
@@ -5603,6 +5695,7 @@
         </is>
       </c>
       <c r="L76" s="7" t="inlineStr"/>
+      <c r="M76" s="7" t="inlineStr"/>
     </row>
     <row r="77" ht="120" customHeight="1">
       <c r="A77" s="9" t="n">
@@ -5659,6 +5752,7 @@
         </is>
       </c>
       <c r="L77" s="9" t="inlineStr"/>
+      <c r="M77" s="9" t="inlineStr"/>
     </row>
     <row r="78" ht="120" customHeight="1">
       <c r="A78" s="7" t="n">
@@ -5715,6 +5809,7 @@
         </is>
       </c>
       <c r="L78" s="7" t="inlineStr"/>
+      <c r="M78" s="7" t="inlineStr"/>
     </row>
     <row r="79" ht="120" customHeight="1">
       <c r="A79" s="9" t="n">
@@ -5771,6 +5866,7 @@
         </is>
       </c>
       <c r="L79" s="9" t="inlineStr"/>
+      <c r="M79" s="9" t="inlineStr"/>
     </row>
     <row r="80" ht="120" customHeight="1">
       <c r="A80" s="7" t="n">
@@ -5827,6 +5923,7 @@
         </is>
       </c>
       <c r="L80" s="7" t="inlineStr"/>
+      <c r="M80" s="7" t="inlineStr"/>
     </row>
     <row r="81" ht="120" customHeight="1">
       <c r="A81" s="9" t="n">
@@ -5883,6 +5980,7 @@
         </is>
       </c>
       <c r="L81" s="9" t="inlineStr"/>
+      <c r="M81" s="9" t="inlineStr"/>
     </row>
     <row r="82" ht="120" customHeight="1">
       <c r="A82" s="7" t="n">
@@ -5939,6 +6037,7 @@
         </is>
       </c>
       <c r="L82" s="7" t="inlineStr"/>
+      <c r="M82" s="7" t="inlineStr"/>
     </row>
     <row r="83" ht="120" customHeight="1">
       <c r="A83" s="9" t="n">
@@ -5995,6 +6094,7 @@
         </is>
       </c>
       <c r="L83" s="9" t="inlineStr"/>
+      <c r="M83" s="9" t="inlineStr"/>
     </row>
     <row r="84" ht="120" customHeight="1">
       <c r="A84" s="7" t="n">
@@ -6051,6 +6151,7 @@
         </is>
       </c>
       <c r="L84" s="7" t="inlineStr"/>
+      <c r="M84" s="7" t="inlineStr"/>
     </row>
     <row r="85" ht="120" customHeight="1">
       <c r="A85" s="9" t="n">
@@ -6107,6 +6208,7 @@
         </is>
       </c>
       <c r="L85" s="9" t="inlineStr"/>
+      <c r="M85" s="9" t="inlineStr"/>
     </row>
     <row r="86" ht="120" customHeight="1">
       <c r="A86" s="7" t="n">
@@ -6163,6 +6265,7 @@
         </is>
       </c>
       <c r="L86" s="7" t="inlineStr"/>
+      <c r="M86" s="7" t="inlineStr"/>
     </row>
     <row r="87" ht="120" customHeight="1">
       <c r="A87" s="9" t="n">
@@ -6219,6 +6322,7 @@
         </is>
       </c>
       <c r="L87" s="9" t="inlineStr"/>
+      <c r="M87" s="9" t="inlineStr"/>
     </row>
     <row r="88" ht="120" customHeight="1">
       <c r="A88" s="7" t="n">
@@ -6275,6 +6379,7 @@
         </is>
       </c>
       <c r="L88" s="7" t="inlineStr"/>
+      <c r="M88" s="7" t="inlineStr"/>
     </row>
     <row r="89" ht="120" customHeight="1">
       <c r="A89" s="9" t="n">
@@ -6331,6 +6436,7 @@
         </is>
       </c>
       <c r="L89" s="9" t="inlineStr"/>
+      <c r="M89" s="9" t="inlineStr"/>
     </row>
     <row r="90" ht="120" customHeight="1">
       <c r="A90" s="7" t="n">
@@ -6387,6 +6493,7 @@
         </is>
       </c>
       <c r="L90" s="7" t="inlineStr"/>
+      <c r="M90" s="7" t="inlineStr"/>
     </row>
     <row r="91" ht="120" customHeight="1">
       <c r="A91" s="9" t="n">
@@ -6443,6 +6550,7 @@
         </is>
       </c>
       <c r="L91" s="9" t="inlineStr"/>
+      <c r="M91" s="9" t="inlineStr"/>
     </row>
     <row r="92" ht="120" customHeight="1">
       <c r="A92" s="7" t="n">
@@ -6499,6 +6607,7 @@
         </is>
       </c>
       <c r="L92" s="7" t="inlineStr"/>
+      <c r="M92" s="7" t="inlineStr"/>
     </row>
     <row r="93" ht="120" customHeight="1">
       <c r="A93" s="9" t="n">
@@ -6555,6 +6664,7 @@
         </is>
       </c>
       <c r="L93" s="9" t="inlineStr"/>
+      <c r="M93" s="9" t="inlineStr"/>
     </row>
     <row r="94" ht="120" customHeight="1">
       <c r="A94" s="7" t="n">
@@ -6611,6 +6721,7 @@
         </is>
       </c>
       <c r="L94" s="7" t="inlineStr"/>
+      <c r="M94" s="7" t="inlineStr"/>
     </row>
     <row r="95" ht="120" customHeight="1">
       <c r="A95" s="9" t="n">
@@ -6667,6 +6778,7 @@
         </is>
       </c>
       <c r="L95" s="9" t="inlineStr"/>
+      <c r="M95" s="9" t="inlineStr"/>
     </row>
     <row r="96" ht="120" customHeight="1">
       <c r="A96" s="7" t="n">
@@ -6723,6 +6835,7 @@
         </is>
       </c>
       <c r="L96" s="7" t="inlineStr"/>
+      <c r="M96" s="7" t="inlineStr"/>
     </row>
     <row r="97" ht="120" customHeight="1">
       <c r="A97" s="9" t="n">
@@ -6779,6 +6892,7 @@
         </is>
       </c>
       <c r="L97" s="9" t="inlineStr"/>
+      <c r="M97" s="9" t="inlineStr"/>
     </row>
     <row r="98" ht="120" customHeight="1">
       <c r="A98" s="7" t="n">
@@ -6835,6 +6949,7 @@
         </is>
       </c>
       <c r="L98" s="7" t="inlineStr"/>
+      <c r="M98" s="7" t="inlineStr"/>
     </row>
     <row r="99" ht="120" customHeight="1">
       <c r="A99" s="9" t="n">
@@ -6891,6 +7006,7 @@
         </is>
       </c>
       <c r="L99" s="9" t="inlineStr"/>
+      <c r="M99" s="9" t="inlineStr"/>
     </row>
     <row r="100" ht="120" customHeight="1">
       <c r="A100" s="7" t="n">
@@ -6947,6 +7063,7 @@
         </is>
       </c>
       <c r="L100" s="7" t="inlineStr"/>
+      <c r="M100" s="7" t="inlineStr"/>
     </row>
     <row r="101" ht="120" customHeight="1">
       <c r="A101" s="9" t="n">
@@ -7003,6 +7120,7 @@
         </is>
       </c>
       <c r="L101" s="9" t="inlineStr"/>
+      <c r="M101" s="9" t="inlineStr"/>
     </row>
     <row r="102" ht="120" customHeight="1">
       <c r="A102" s="7" t="n">
@@ -7059,6 +7177,7 @@
         </is>
       </c>
       <c r="L102" s="7" t="inlineStr"/>
+      <c r="M102" s="7" t="inlineStr"/>
     </row>
     <row r="103" ht="120" customHeight="1">
       <c r="A103" s="9" t="n">
@@ -7115,6 +7234,7 @@
         </is>
       </c>
       <c r="L103" s="9" t="inlineStr"/>
+      <c r="M103" s="9" t="inlineStr"/>
     </row>
     <row r="104" ht="120" customHeight="1">
       <c r="A104" s="7" t="n">
@@ -7171,6 +7291,7 @@
         </is>
       </c>
       <c r="L104" s="7" t="inlineStr"/>
+      <c r="M104" s="7" t="inlineStr"/>
     </row>
     <row r="105" ht="120" customHeight="1">
       <c r="A105" s="9" t="n">
@@ -7227,6 +7348,7 @@
         </is>
       </c>
       <c r="L105" s="9" t="inlineStr"/>
+      <c r="M105" s="9" t="inlineStr"/>
     </row>
     <row r="106" ht="120" customHeight="1">
       <c r="A106" s="7" t="n">
@@ -7283,6 +7405,7 @@
         </is>
       </c>
       <c r="L106" s="7" t="inlineStr"/>
+      <c r="M106" s="7" t="inlineStr"/>
     </row>
     <row r="107" ht="120" customHeight="1">
       <c r="A107" s="9" t="n">
@@ -7339,6 +7462,7 @@
         </is>
       </c>
       <c r="L107" s="9" t="inlineStr"/>
+      <c r="M107" s="9" t="inlineStr"/>
     </row>
     <row r="108" ht="120" customHeight="1">
       <c r="A108" s="7" t="n">
@@ -7395,6 +7519,7 @@
         </is>
       </c>
       <c r="L108" s="7" t="inlineStr"/>
+      <c r="M108" s="7" t="inlineStr"/>
     </row>
     <row r="109" ht="120" customHeight="1">
       <c r="A109" s="9" t="n">
@@ -7451,6 +7576,7 @@
         </is>
       </c>
       <c r="L109" s="9" t="inlineStr"/>
+      <c r="M109" s="9" t="inlineStr"/>
     </row>
     <row r="110" ht="120" customHeight="1">
       <c r="A110" s="7" t="n">
@@ -7507,6 +7633,7 @@
         </is>
       </c>
       <c r="L110" s="7" t="inlineStr"/>
+      <c r="M110" s="7" t="inlineStr"/>
     </row>
     <row r="111" ht="120" customHeight="1">
       <c r="A111" s="9" t="n">
@@ -7563,6 +7690,7 @@
         </is>
       </c>
       <c r="L111" s="9" t="inlineStr"/>
+      <c r="M111" s="9" t="inlineStr"/>
     </row>
     <row r="112" ht="120" customHeight="1">
       <c r="A112" s="7" t="n">
@@ -7619,6 +7747,7 @@
         </is>
       </c>
       <c r="L112" s="7" t="inlineStr"/>
+      <c r="M112" s="7" t="inlineStr"/>
     </row>
     <row r="113" ht="120" customHeight="1">
       <c r="A113" s="9" t="n">
@@ -7675,6 +7804,7 @@
         </is>
       </c>
       <c r="L113" s="9" t="inlineStr"/>
+      <c r="M113" s="9" t="inlineStr"/>
     </row>
     <row r="114" ht="120" customHeight="1">
       <c r="A114" s="7" t="n">
@@ -7731,6 +7861,7 @@
         </is>
       </c>
       <c r="L114" s="7" t="inlineStr"/>
+      <c r="M114" s="7" t="inlineStr"/>
     </row>
     <row r="115" ht="120" customHeight="1">
       <c r="A115" s="9" t="n">
@@ -7787,6 +7918,7 @@
         </is>
       </c>
       <c r="L115" s="9" t="inlineStr"/>
+      <c r="M115" s="9" t="inlineStr"/>
     </row>
     <row r="116" ht="120" customHeight="1">
       <c r="A116" s="7" t="n">
@@ -7843,6 +7975,7 @@
         </is>
       </c>
       <c r="L116" s="7" t="inlineStr"/>
+      <c r="M116" s="7" t="inlineStr"/>
     </row>
     <row r="117" ht="120" customHeight="1">
       <c r="A117" s="9" t="n">
@@ -7899,6 +8032,7 @@
         </is>
       </c>
       <c r="L117" s="9" t="inlineStr"/>
+      <c r="M117" s="9" t="inlineStr"/>
     </row>
     <row r="118" ht="120" customHeight="1">
       <c r="A118" s="7" t="n">
@@ -7955,6 +8089,7 @@
         </is>
       </c>
       <c r="L118" s="7" t="inlineStr"/>
+      <c r="M118" s="7" t="inlineStr"/>
     </row>
     <row r="119" ht="120" customHeight="1">
       <c r="A119" s="9" t="n">
@@ -8011,6 +8146,7 @@
         </is>
       </c>
       <c r="L119" s="9" t="inlineStr"/>
+      <c r="M119" s="9" t="inlineStr"/>
     </row>
     <row r="120" ht="120" customHeight="1">
       <c r="A120" s="7" t="n">
@@ -8067,6 +8203,7 @@
         </is>
       </c>
       <c r="L120" s="7" t="inlineStr"/>
+      <c r="M120" s="7" t="inlineStr"/>
     </row>
     <row r="121" ht="120" customHeight="1">
       <c r="A121" s="9" t="n">
@@ -8123,6 +8260,7 @@
         </is>
       </c>
       <c r="L121" s="9" t="inlineStr"/>
+      <c r="M121" s="9" t="inlineStr"/>
     </row>
     <row r="122" ht="120" customHeight="1">
       <c r="A122" s="7" t="n">
@@ -8179,6 +8317,7 @@
         </is>
       </c>
       <c r="L122" s="7" t="inlineStr"/>
+      <c r="M122" s="7" t="inlineStr"/>
     </row>
     <row r="123" ht="120" customHeight="1">
       <c r="A123" s="9" t="n">
@@ -8235,6 +8374,7 @@
         </is>
       </c>
       <c r="L123" s="9" t="inlineStr"/>
+      <c r="M123" s="9" t="inlineStr"/>
     </row>
     <row r="124" ht="120" customHeight="1">
       <c r="A124" s="7" t="n">
@@ -8291,6 +8431,7 @@
         </is>
       </c>
       <c r="L124" s="7" t="inlineStr"/>
+      <c r="M124" s="7" t="inlineStr"/>
     </row>
     <row r="125" ht="120" customHeight="1">
       <c r="A125" s="9" t="n">
@@ -8347,6 +8488,7 @@
         </is>
       </c>
       <c r="L125" s="9" t="inlineStr"/>
+      <c r="M125" s="9" t="inlineStr"/>
     </row>
     <row r="126" ht="120" customHeight="1">
       <c r="A126" s="7" t="n">
@@ -8403,6 +8545,7 @@
         </is>
       </c>
       <c r="L126" s="7" t="inlineStr"/>
+      <c r="M126" s="7" t="inlineStr"/>
     </row>
     <row r="127" ht="120" customHeight="1">
       <c r="A127" s="9" t="n">
@@ -8459,6 +8602,7 @@
         </is>
       </c>
       <c r="L127" s="9" t="inlineStr"/>
+      <c r="M127" s="9" t="inlineStr"/>
     </row>
     <row r="128" ht="120" customHeight="1">
       <c r="A128" s="7" t="n">
@@ -8515,6 +8659,7 @@
         </is>
       </c>
       <c r="L128" s="7" t="inlineStr"/>
+      <c r="M128" s="7" t="inlineStr"/>
     </row>
     <row r="129" ht="120" customHeight="1">
       <c r="A129" s="9" t="n">
@@ -8571,6 +8716,7 @@
         </is>
       </c>
       <c r="L129" s="9" t="inlineStr"/>
+      <c r="M129" s="9" t="inlineStr"/>
     </row>
     <row r="130" ht="120" customHeight="1">
       <c r="A130" s="7" t="n">
@@ -8627,6 +8773,7 @@
         </is>
       </c>
       <c r="L130" s="7" t="inlineStr"/>
+      <c r="M130" s="7" t="inlineStr"/>
     </row>
     <row r="131" ht="120" customHeight="1">
       <c r="A131" s="9" t="n">
@@ -8683,6 +8830,7 @@
         </is>
       </c>
       <c r="L131" s="9" t="inlineStr"/>
+      <c r="M131" s="9" t="inlineStr"/>
     </row>
     <row r="132" ht="120" customHeight="1">
       <c r="A132" s="7" t="n">
@@ -8739,6 +8887,7 @@
         </is>
       </c>
       <c r="L132" s="7" t="inlineStr"/>
+      <c r="M132" s="7" t="inlineStr"/>
     </row>
     <row r="133" ht="120" customHeight="1">
       <c r="A133" s="9" t="n">
@@ -8795,6 +8944,7 @@
         </is>
       </c>
       <c r="L133" s="9" t="inlineStr"/>
+      <c r="M133" s="9" t="inlineStr"/>
     </row>
     <row r="134" ht="120" customHeight="1">
       <c r="A134" s="7" t="n">
@@ -8851,6 +9001,7 @@
         </is>
       </c>
       <c r="L134" s="7" t="inlineStr"/>
+      <c r="M134" s="7" t="inlineStr"/>
     </row>
     <row r="135" ht="120" customHeight="1">
       <c r="A135" s="9" t="n">
@@ -8907,6 +9058,7 @@
         </is>
       </c>
       <c r="L135" s="9" t="inlineStr"/>
+      <c r="M135" s="9" t="inlineStr"/>
     </row>
     <row r="136" ht="120" customHeight="1">
       <c r="A136" s="7" t="n">
@@ -8963,6 +9115,7 @@
         </is>
       </c>
       <c r="L136" s="7" t="inlineStr"/>
+      <c r="M136" s="7" t="inlineStr"/>
     </row>
     <row r="137" ht="120" customHeight="1">
       <c r="A137" s="9" t="n">
@@ -9019,6 +9172,7 @@
         </is>
       </c>
       <c r="L137" s="9" t="inlineStr"/>
+      <c r="M137" s="9" t="inlineStr"/>
     </row>
     <row r="138" ht="120" customHeight="1">
       <c r="A138" s="7" t="n">
@@ -9075,6 +9229,7 @@
         </is>
       </c>
       <c r="L138" s="7" t="inlineStr"/>
+      <c r="M138" s="7" t="inlineStr"/>
     </row>
     <row r="139" ht="120" customHeight="1">
       <c r="A139" s="9" t="n">
@@ -9131,6 +9286,7 @@
         </is>
       </c>
       <c r="L139" s="9" t="inlineStr"/>
+      <c r="M139" s="9" t="inlineStr"/>
     </row>
     <row r="140" ht="120" customHeight="1">
       <c r="A140" s="7" t="n">
@@ -9187,6 +9343,7 @@
         </is>
       </c>
       <c r="L140" s="7" t="inlineStr"/>
+      <c r="M140" s="7" t="inlineStr"/>
     </row>
     <row r="141" ht="120" customHeight="1">
       <c r="A141" s="9" t="n">
@@ -9243,6 +9400,7 @@
         </is>
       </c>
       <c r="L141" s="9" t="inlineStr"/>
+      <c r="M141" s="9" t="inlineStr"/>
     </row>
     <row r="142" ht="120" customHeight="1">
       <c r="A142" s="7" t="n">
@@ -9299,6 +9457,7 @@
         </is>
       </c>
       <c r="L142" s="7" t="inlineStr"/>
+      <c r="M142" s="7" t="inlineStr"/>
     </row>
     <row r="143" ht="120" customHeight="1">
       <c r="A143" s="9" t="n">
@@ -9355,6 +9514,7 @@
         </is>
       </c>
       <c r="L143" s="9" t="inlineStr"/>
+      <c r="M143" s="9" t="inlineStr"/>
     </row>
     <row r="144" ht="120" customHeight="1">
       <c r="A144" s="7" t="n">
@@ -9411,6 +9571,7 @@
         </is>
       </c>
       <c r="L144" s="7" t="inlineStr"/>
+      <c r="M144" s="7" t="inlineStr"/>
     </row>
     <row r="145" ht="120" customHeight="1">
       <c r="A145" s="9" t="n">
@@ -9467,6 +9628,7 @@
         </is>
       </c>
       <c r="L145" s="9" t="inlineStr"/>
+      <c r="M145" s="9" t="inlineStr"/>
     </row>
     <row r="146" ht="120" customHeight="1">
       <c r="A146" s="7" t="n">
@@ -9523,6 +9685,7 @@
         </is>
       </c>
       <c r="L146" s="7" t="inlineStr"/>
+      <c r="M146" s="7" t="inlineStr"/>
     </row>
     <row r="147" ht="120" customHeight="1">
       <c r="A147" s="9" t="n">
@@ -9579,6 +9742,7 @@
         </is>
       </c>
       <c r="L147" s="9" t="inlineStr"/>
+      <c r="M147" s="9" t="inlineStr"/>
     </row>
     <row r="148" ht="120" customHeight="1">
       <c r="A148" s="7" t="n">
@@ -9635,6 +9799,7 @@
         </is>
       </c>
       <c r="L148" s="7" t="inlineStr"/>
+      <c r="M148" s="7" t="inlineStr"/>
     </row>
     <row r="149" ht="120" customHeight="1">
       <c r="A149" s="9" t="n">
@@ -9691,6 +9856,7 @@
         </is>
       </c>
       <c r="L149" s="9" t="inlineStr"/>
+      <c r="M149" s="9" t="inlineStr"/>
     </row>
     <row r="150" ht="120" customHeight="1">
       <c r="A150" s="7" t="n">
@@ -9747,6 +9913,7 @@
         </is>
       </c>
       <c r="L150" s="7" t="inlineStr"/>
+      <c r="M150" s="7" t="inlineStr"/>
     </row>
     <row r="151" ht="120" customHeight="1">
       <c r="A151" s="9" t="n">
@@ -9803,6 +9970,7 @@
         </is>
       </c>
       <c r="L151" s="9" t="inlineStr"/>
+      <c r="M151" s="9" t="inlineStr"/>
     </row>
     <row r="152" ht="120" customHeight="1">
       <c r="A152" s="7" t="n">
@@ -9859,6 +10027,7 @@
         </is>
       </c>
       <c r="L152" s="7" t="inlineStr"/>
+      <c r="M152" s="7" t="inlineStr"/>
     </row>
     <row r="153" ht="120" customHeight="1">
       <c r="A153" s="9" t="n">
@@ -9915,6 +10084,7 @@
         </is>
       </c>
       <c r="L153" s="9" t="inlineStr"/>
+      <c r="M153" s="9" t="inlineStr"/>
     </row>
     <row r="154" ht="120" customHeight="1">
       <c r="A154" s="7" t="n">
@@ -9971,6 +10141,7 @@
         </is>
       </c>
       <c r="L154" s="7" t="inlineStr"/>
+      <c r="M154" s="7" t="inlineStr"/>
     </row>
     <row r="155" ht="120" customHeight="1">
       <c r="A155" s="9" t="n">
@@ -10027,6 +10198,7 @@
         </is>
       </c>
       <c r="L155" s="9" t="inlineStr"/>
+      <c r="M155" s="9" t="inlineStr"/>
     </row>
     <row r="156" ht="120" customHeight="1">
       <c r="A156" s="7" t="n">
@@ -10083,6 +10255,7 @@
         </is>
       </c>
       <c r="L156" s="7" t="inlineStr"/>
+      <c r="M156" s="7" t="inlineStr"/>
     </row>
     <row r="157" ht="120" customHeight="1">
       <c r="A157" s="9" t="n">
@@ -10139,6 +10312,7 @@
         </is>
       </c>
       <c r="L157" s="9" t="inlineStr"/>
+      <c r="M157" s="9" t="inlineStr"/>
     </row>
     <row r="158" ht="120" customHeight="1">
       <c r="A158" s="7" t="n">
@@ -10195,6 +10369,7 @@
         </is>
       </c>
       <c r="L158" s="7" t="inlineStr"/>
+      <c r="M158" s="7" t="inlineStr"/>
     </row>
     <row r="159" ht="120" customHeight="1">
       <c r="A159" s="9" t="n">
@@ -10251,6 +10426,7 @@
         </is>
       </c>
       <c r="L159" s="9" t="inlineStr"/>
+      <c r="M159" s="9" t="inlineStr"/>
     </row>
     <row r="160" ht="120" customHeight="1">
       <c r="A160" s="7" t="n">
@@ -10307,6 +10483,7 @@
         </is>
       </c>
       <c r="L160" s="7" t="inlineStr"/>
+      <c r="M160" s="7" t="inlineStr"/>
     </row>
     <row r="161" ht="120" customHeight="1">
       <c r="A161" s="9" t="n">
@@ -10363,6 +10540,7 @@
         </is>
       </c>
       <c r="L161" s="9" t="inlineStr"/>
+      <c r="M161" s="9" t="inlineStr"/>
     </row>
     <row r="162" ht="120" customHeight="1">
       <c r="A162" s="7" t="n">
@@ -10419,6 +10597,7 @@
         </is>
       </c>
       <c r="L162" s="7" t="inlineStr"/>
+      <c r="M162" s="7" t="inlineStr"/>
     </row>
     <row r="163" ht="120" customHeight="1">
       <c r="A163" s="9" t="n">
@@ -10475,6 +10654,7 @@
         </is>
       </c>
       <c r="L163" s="9" t="inlineStr"/>
+      <c r="M163" s="9" t="inlineStr"/>
     </row>
     <row r="164" ht="120" customHeight="1">
       <c r="A164" s="7" t="n">
@@ -10531,6 +10711,7 @@
         </is>
       </c>
       <c r="L164" s="7" t="inlineStr"/>
+      <c r="M164" s="7" t="inlineStr"/>
     </row>
     <row r="165" ht="120" customHeight="1">
       <c r="A165" s="9" t="n">
@@ -10587,6 +10768,7 @@
         </is>
       </c>
       <c r="L165" s="9" t="inlineStr"/>
+      <c r="M165" s="9" t="inlineStr"/>
     </row>
     <row r="166" ht="120" customHeight="1">
       <c r="A166" s="7" t="n">
@@ -10643,6 +10825,7 @@
         </is>
       </c>
       <c r="L166" s="7" t="inlineStr"/>
+      <c r="M166" s="7" t="inlineStr"/>
     </row>
     <row r="167" ht="120" customHeight="1">
       <c r="A167" s="9" t="n">
@@ -10699,6 +10882,7 @@
         </is>
       </c>
       <c r="L167" s="9" t="inlineStr"/>
+      <c r="M167" s="9" t="inlineStr"/>
     </row>
     <row r="168" ht="120" customHeight="1">
       <c r="A168" s="7" t="n">
@@ -10755,6 +10939,7 @@
         </is>
       </c>
       <c r="L168" s="7" t="inlineStr"/>
+      <c r="M168" s="7" t="inlineStr"/>
     </row>
     <row r="169" ht="120" customHeight="1">
       <c r="A169" s="9" t="n">
@@ -10811,6 +10996,7 @@
         </is>
       </c>
       <c r="L169" s="9" t="inlineStr"/>
+      <c r="M169" s="9" t="inlineStr"/>
     </row>
     <row r="170" ht="120" customHeight="1">
       <c r="A170" s="7" t="n">
@@ -10867,6 +11053,7 @@
         </is>
       </c>
       <c r="L170" s="7" t="inlineStr"/>
+      <c r="M170" s="7" t="inlineStr"/>
     </row>
     <row r="171" ht="120" customHeight="1">
       <c r="A171" s="9" t="n">
@@ -10923,6 +11110,7 @@
         </is>
       </c>
       <c r="L171" s="9" t="inlineStr"/>
+      <c r="M171" s="9" t="inlineStr"/>
     </row>
     <row r="172" ht="120" customHeight="1">
       <c r="A172" s="7" t="n">
@@ -10979,6 +11167,7 @@
         </is>
       </c>
       <c r="L172" s="7" t="inlineStr"/>
+      <c r="M172" s="7" t="inlineStr"/>
     </row>
     <row r="173" ht="120" customHeight="1">
       <c r="A173" s="9" t="n">
@@ -11035,6 +11224,7 @@
         </is>
       </c>
       <c r="L173" s="9" t="inlineStr"/>
+      <c r="M173" s="9" t="inlineStr"/>
     </row>
     <row r="174" ht="120" customHeight="1">
       <c r="A174" s="7" t="n">
@@ -11091,6 +11281,7 @@
         </is>
       </c>
       <c r="L174" s="7" t="inlineStr"/>
+      <c r="M174" s="7" t="inlineStr"/>
     </row>
     <row r="175" ht="120" customHeight="1">
       <c r="A175" s="9" t="n">
@@ -11147,6 +11338,7 @@
         </is>
       </c>
       <c r="L175" s="9" t="inlineStr"/>
+      <c r="M175" s="9" t="inlineStr"/>
     </row>
     <row r="176" ht="120" customHeight="1">
       <c r="A176" s="7" t="n">
@@ -11203,6 +11395,7 @@
         </is>
       </c>
       <c r="L176" s="7" t="inlineStr"/>
+      <c r="M176" s="7" t="inlineStr"/>
     </row>
     <row r="177" ht="120" customHeight="1">
       <c r="A177" s="9" t="n">
@@ -11259,6 +11452,7 @@
         </is>
       </c>
       <c r="L177" s="9" t="inlineStr"/>
+      <c r="M177" s="9" t="inlineStr"/>
     </row>
     <row r="178" ht="120" customHeight="1">
       <c r="A178" s="7" t="n">
@@ -11315,6 +11509,7 @@
         </is>
       </c>
       <c r="L178" s="7" t="inlineStr"/>
+      <c r="M178" s="7" t="inlineStr"/>
     </row>
     <row r="179" ht="120" customHeight="1">
       <c r="A179" s="9" t="n">
@@ -11371,6 +11566,7 @@
         </is>
       </c>
       <c r="L179" s="9" t="inlineStr"/>
+      <c r="M179" s="9" t="inlineStr"/>
     </row>
     <row r="180" ht="120" customHeight="1">
       <c r="A180" s="7" t="n">
@@ -11427,6 +11623,7 @@
         </is>
       </c>
       <c r="L180" s="7" t="inlineStr"/>
+      <c r="M180" s="7" t="inlineStr"/>
     </row>
     <row r="181" ht="120" customHeight="1">
       <c r="A181" s="9" t="n">
@@ -11483,6 +11680,7 @@
         </is>
       </c>
       <c r="L181" s="9" t="inlineStr"/>
+      <c r="M181" s="9" t="inlineStr"/>
     </row>
     <row r="182" ht="120" customHeight="1">
       <c r="A182" s="7" t="n">
@@ -11539,6 +11737,7 @@
         </is>
       </c>
       <c r="L182" s="7" t="inlineStr"/>
+      <c r="M182" s="7" t="inlineStr"/>
     </row>
     <row r="183" ht="120" customHeight="1">
       <c r="A183" s="9" t="n">
@@ -11595,6 +11794,7 @@
         </is>
       </c>
       <c r="L183" s="9" t="inlineStr"/>
+      <c r="M183" s="9" t="inlineStr"/>
     </row>
     <row r="184" ht="120" customHeight="1">
       <c r="A184" s="7" t="n">
@@ -11651,6 +11851,7 @@
         </is>
       </c>
       <c r="L184" s="7" t="inlineStr"/>
+      <c r="M184" s="7" t="inlineStr"/>
     </row>
     <row r="185" ht="120" customHeight="1">
       <c r="A185" s="9" t="n">
@@ -11707,6 +11908,7 @@
         </is>
       </c>
       <c r="L185" s="9" t="inlineStr"/>
+      <c r="M185" s="9" t="inlineStr"/>
     </row>
     <row r="186" ht="120" customHeight="1">
       <c r="A186" s="7" t="n">
@@ -11763,6 +11965,7 @@
         </is>
       </c>
       <c r="L186" s="7" t="inlineStr"/>
+      <c r="M186" s="7" t="inlineStr"/>
     </row>
     <row r="187" ht="120" customHeight="1">
       <c r="A187" s="9" t="n">
@@ -11819,6 +12022,7 @@
         </is>
       </c>
       <c r="L187" s="9" t="inlineStr"/>
+      <c r="M187" s="9" t="inlineStr"/>
     </row>
     <row r="188" ht="120" customHeight="1">
       <c r="A188" s="7" t="n">
@@ -11875,6 +12079,7 @@
         </is>
       </c>
       <c r="L188" s="7" t="inlineStr"/>
+      <c r="M188" s="7" t="inlineStr"/>
     </row>
     <row r="189" ht="120" customHeight="1">
       <c r="A189" s="9" t="n">
@@ -11931,6 +12136,7 @@
         </is>
       </c>
       <c r="L189" s="9" t="inlineStr"/>
+      <c r="M189" s="9" t="inlineStr"/>
     </row>
     <row r="190" ht="120" customHeight="1">
       <c r="A190" s="7" t="n">
@@ -11987,6 +12193,7 @@
         </is>
       </c>
       <c r="L190" s="7" t="inlineStr"/>
+      <c r="M190" s="7" t="inlineStr"/>
     </row>
     <row r="191" ht="120" customHeight="1">
       <c r="A191" s="9" t="n">
@@ -12043,6 +12250,7 @@
         </is>
       </c>
       <c r="L191" s="9" t="inlineStr"/>
+      <c r="M191" s="9" t="inlineStr"/>
     </row>
     <row r="192" ht="120" customHeight="1">
       <c r="A192" s="7" t="n">
@@ -12073,24 +12281,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G192" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G192" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H192" s="7" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I192" s="7" t="inlineStr">
         <is>
-          <t>a small round painted badge showing a tall rooftop with an upward arrow, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a tall rooftop with an upward arrow, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J192" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K192" s="7" t="inlineStr">
@@ -12099,6 +12307,7 @@
         </is>
       </c>
       <c r="L192" s="7" t="inlineStr"/>
+      <c r="M192" s="7" t="inlineStr"/>
     </row>
     <row r="193" ht="120" customHeight="1">
       <c r="A193" s="9" t="n">
@@ -12129,24 +12338,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G193" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G193" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H193" s="9" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I193" s="9" t="inlineStr">
         <is>
-          <t>a small round painted badge showing a rooftop with a wall blocking wind swirls, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a rooftop with a wall blocking wind swirls, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J193" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K193" s="9" t="inlineStr">
@@ -12155,6 +12364,7 @@
         </is>
       </c>
       <c r="L193" s="9" t="inlineStr"/>
+      <c r="M193" s="9" t="inlineStr"/>
     </row>
     <row r="194" ht="120" customHeight="1">
       <c r="A194" s="7" t="n">
@@ -12185,24 +12395,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G194" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G194" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H194" s="7" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I194" s="7" t="inlineStr">
         <is>
-          <t>a small round painted badge showing a wind gust swirl with an arrow, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a wind gust swirl with an arrow, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J194" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K194" s="7" t="inlineStr">
@@ -12211,6 +12421,7 @@
         </is>
       </c>
       <c r="L194" s="7" t="inlineStr"/>
+      <c r="M194" s="7" t="inlineStr"/>
     </row>
     <row r="195" ht="120" customHeight="1">
       <c r="A195" s="9" t="n">
@@ -12241,24 +12452,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G195" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G195" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H195" s="9" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I195" s="9" t="inlineStr">
         <is>
-          <t>a small round painted badge showing a small wooden supply crate with a kite symbol, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a small wooden supply crate with a kite symbol, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J195" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K195" s="9" t="inlineStr">
@@ -12267,6 +12478,7 @@
         </is>
       </c>
       <c r="L195" s="9" t="inlineStr"/>
+      <c r="M195" s="9" t="inlineStr"/>
     </row>
     <row r="196" ht="120" customHeight="1">
       <c r="A196" s="7" t="n">
@@ -12297,24 +12509,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G196" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G196" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I196" s="7" t="inlineStr">
         <is>
-          <t>a small round painted badge showing a rooftop edge with a caution stripe, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a rooftop edge with a caution stripe, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J196" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K196" s="7" t="inlineStr">
@@ -12323,6 +12535,7 @@
         </is>
       </c>
       <c r="L196" s="7" t="inlineStr"/>
+      <c r="M196" s="7" t="inlineStr"/>
     </row>
     <row r="197" ht="120" customHeight="1">
       <c r="A197" s="9" t="n">
@@ -12353,24 +12566,24 @@
           <t>Roof select screen, map labels</t>
         </is>
       </c>
-      <c r="G197" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G197" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H197" s="9" t="inlineStr">
         <is>
-          <t>Tiny badge – must read at 40 px. Simple shape.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Must read at 40 px.</t>
         </is>
       </c>
       <c r="I197" s="9" t="inlineStr">
         <is>
-          <t>a small round painted badge showing tangled overhead cables (warning), single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of tangled overhead cables (warning), pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J197" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K197" s="9" t="inlineStr">
@@ -12379,6 +12592,7 @@
         </is>
       </c>
       <c r="L197" s="9" t="inlineStr"/>
+      <c r="M197" s="9" t="inlineStr"/>
     </row>
     <row r="198" ht="120" customHeight="1">
       <c r="A198" s="7" t="n">
@@ -12435,6 +12649,7 @@
         </is>
       </c>
       <c r="L198" s="7" t="inlineStr"/>
+      <c r="M198" s="7" t="inlineStr"/>
     </row>
     <row r="199" ht="120" customHeight="1">
       <c r="A199" s="9" t="n">
@@ -12491,6 +12706,7 @@
         </is>
       </c>
       <c r="L199" s="9" t="inlineStr"/>
+      <c r="M199" s="9" t="inlineStr"/>
     </row>
     <row r="200" ht="120" customHeight="1">
       <c r="A200" s="7" t="n">
@@ -12547,6 +12763,7 @@
         </is>
       </c>
       <c r="L200" s="7" t="inlineStr"/>
+      <c r="M200" s="7" t="inlineStr"/>
     </row>
     <row r="201" ht="120" customHeight="1">
       <c r="A201" s="9" t="n">
@@ -12603,6 +12820,7 @@
         </is>
       </c>
       <c r="L201" s="9" t="inlineStr"/>
+      <c r="M201" s="9" t="inlineStr"/>
     </row>
     <row r="202" ht="120" customHeight="1">
       <c r="A202" s="7" t="n">
@@ -12659,6 +12877,7 @@
         </is>
       </c>
       <c r="L202" s="7" t="inlineStr"/>
+      <c r="M202" s="7" t="inlineStr"/>
     </row>
     <row r="203" ht="120" customHeight="1">
       <c r="A203" s="9" t="n">
@@ -12715,6 +12934,7 @@
         </is>
       </c>
       <c r="L203" s="9" t="inlineStr"/>
+      <c r="M203" s="9" t="inlineStr"/>
     </row>
     <row r="204" ht="120" customHeight="1">
       <c r="A204" s="7" t="n">
@@ -12771,6 +12991,7 @@
         </is>
       </c>
       <c r="L204" s="7" t="inlineStr"/>
+      <c r="M204" s="7" t="inlineStr"/>
     </row>
     <row r="205" ht="120" customHeight="1">
       <c r="A205" s="9" t="n">
@@ -12827,6 +13048,7 @@
         </is>
       </c>
       <c r="L205" s="9" t="inlineStr"/>
+      <c r="M205" s="9" t="inlineStr"/>
     </row>
     <row r="206" ht="120" customHeight="1">
       <c r="A206" s="7" t="n">
@@ -12883,6 +13105,7 @@
         </is>
       </c>
       <c r="L206" s="7" t="inlineStr"/>
+      <c r="M206" s="7" t="inlineStr"/>
     </row>
     <row r="207" ht="120" customHeight="1">
       <c r="A207" s="9" t="n">
@@ -12939,6 +13162,7 @@
         </is>
       </c>
       <c r="L207" s="9" t="inlineStr"/>
+      <c r="M207" s="9" t="inlineStr"/>
     </row>
     <row r="208" ht="120" customHeight="1">
       <c r="A208" s="7" t="n">
@@ -12995,6 +13219,7 @@
         </is>
       </c>
       <c r="L208" s="7" t="inlineStr"/>
+      <c r="M208" s="7" t="inlineStr"/>
     </row>
     <row r="209" ht="120" customHeight="1">
       <c r="A209" s="9" t="n">
@@ -13051,6 +13276,7 @@
         </is>
       </c>
       <c r="L209" s="9" t="inlineStr"/>
+      <c r="M209" s="9" t="inlineStr"/>
     </row>
     <row r="210" ht="120" customHeight="1">
       <c r="A210" s="7" t="n">
@@ -13107,6 +13333,7 @@
         </is>
       </c>
       <c r="L210" s="7" t="inlineStr"/>
+      <c r="M210" s="7" t="inlineStr"/>
     </row>
     <row r="211" ht="120" customHeight="1">
       <c r="A211" s="9" t="n">
@@ -13163,6 +13390,7 @@
         </is>
       </c>
       <c r="L211" s="9" t="inlineStr"/>
+      <c r="M211" s="9" t="inlineStr"/>
     </row>
     <row r="212" ht="120" customHeight="1">
       <c r="A212" s="7" t="n">
@@ -13219,6 +13447,7 @@
         </is>
       </c>
       <c r="L212" s="7" t="inlineStr"/>
+      <c r="M212" s="7" t="inlineStr"/>
     </row>
     <row r="213" ht="120" customHeight="1">
       <c r="A213" s="9" t="n">
@@ -13275,6 +13504,7 @@
         </is>
       </c>
       <c r="L213" s="9" t="inlineStr"/>
+      <c r="M213" s="9" t="inlineStr"/>
     </row>
     <row r="214" ht="120" customHeight="1">
       <c r="A214" s="7" t="n">
@@ -13331,6 +13561,7 @@
         </is>
       </c>
       <c r="L214" s="7" t="inlineStr"/>
+      <c r="M214" s="7" t="inlineStr"/>
     </row>
     <row r="215" ht="120" customHeight="1">
       <c r="A215" s="9" t="n">
@@ -13387,6 +13618,7 @@
         </is>
       </c>
       <c r="L215" s="9" t="inlineStr"/>
+      <c r="M215" s="9" t="inlineStr"/>
     </row>
     <row r="216" ht="120" customHeight="1">
       <c r="A216" s="7" t="n">
@@ -13443,6 +13675,7 @@
         </is>
       </c>
       <c r="L216" s="7" t="inlineStr"/>
+      <c r="M216" s="7" t="inlineStr"/>
     </row>
     <row r="217" ht="120" customHeight="1">
       <c r="A217" s="9" t="n">
@@ -13499,6 +13732,7 @@
         </is>
       </c>
       <c r="L217" s="9" t="inlineStr"/>
+      <c r="M217" s="9" t="inlineStr"/>
     </row>
     <row r="218" ht="120" customHeight="1">
       <c r="A218" s="7" t="n">
@@ -13555,6 +13789,7 @@
         </is>
       </c>
       <c r="L218" s="7" t="inlineStr"/>
+      <c r="M218" s="7" t="inlineStr"/>
     </row>
     <row r="219" ht="120" customHeight="1">
       <c r="A219" s="9" t="n">
@@ -13611,6 +13846,7 @@
         </is>
       </c>
       <c r="L219" s="9" t="inlineStr"/>
+      <c r="M219" s="9" t="inlineStr"/>
     </row>
     <row r="220" ht="120" customHeight="1">
       <c r="A220" s="7" t="n">
@@ -13667,6 +13903,7 @@
         </is>
       </c>
       <c r="L220" s="7" t="inlineStr"/>
+      <c r="M220" s="7" t="inlineStr"/>
     </row>
     <row r="221" ht="120" customHeight="1">
       <c r="A221" s="9" t="n">
@@ -13723,6 +13960,7 @@
         </is>
       </c>
       <c r="L221" s="9" t="inlineStr"/>
+      <c r="M221" s="9" t="inlineStr"/>
     </row>
     <row r="222" ht="120" customHeight="1">
       <c r="A222" s="7" t="n">
@@ -13779,6 +14017,7 @@
         </is>
       </c>
       <c r="L222" s="7" t="inlineStr"/>
+      <c r="M222" s="7" t="inlineStr"/>
     </row>
     <row r="223" ht="120" customHeight="1">
       <c r="A223" s="9" t="n">
@@ -13835,6 +14074,7 @@
         </is>
       </c>
       <c r="L223" s="9" t="inlineStr"/>
+      <c r="M223" s="9" t="inlineStr"/>
     </row>
     <row r="224" ht="120" customHeight="1">
       <c r="A224" s="7" t="n">
@@ -13891,6 +14131,7 @@
         </is>
       </c>
       <c r="L224" s="7" t="inlineStr"/>
+      <c r="M224" s="7" t="inlineStr"/>
     </row>
     <row r="225" ht="120" customHeight="1">
       <c r="A225" s="9" t="n">
@@ -13947,6 +14188,7 @@
         </is>
       </c>
       <c r="L225" s="9" t="inlineStr"/>
+      <c r="M225" s="9" t="inlineStr"/>
     </row>
     <row r="226" ht="120" customHeight="1">
       <c r="A226" s="7" t="n">
@@ -14003,6 +14245,7 @@
         </is>
       </c>
       <c r="L226" s="7" t="inlineStr"/>
+      <c r="M226" s="7" t="inlineStr"/>
     </row>
     <row r="227" ht="120" customHeight="1">
       <c r="A227" s="9" t="n">
@@ -14059,6 +14302,7 @@
         </is>
       </c>
       <c r="L227" s="9" t="inlineStr"/>
+      <c r="M227" s="9" t="inlineStr"/>
     </row>
     <row r="228" ht="120" customHeight="1">
       <c r="A228" s="7" t="n">
@@ -14115,6 +14359,7 @@
         </is>
       </c>
       <c r="L228" s="7" t="inlineStr"/>
+      <c r="M228" s="7" t="inlineStr"/>
     </row>
     <row r="229" ht="120" customHeight="1">
       <c r="A229" s="9" t="n">
@@ -14171,6 +14416,7 @@
         </is>
       </c>
       <c r="L229" s="9" t="inlineStr"/>
+      <c r="M229" s="9" t="inlineStr"/>
     </row>
     <row r="230" ht="120" customHeight="1">
       <c r="A230" s="7" t="n">
@@ -14227,6 +14473,7 @@
         </is>
       </c>
       <c r="L230" s="7" t="inlineStr"/>
+      <c r="M230" s="7" t="inlineStr"/>
     </row>
     <row r="231" ht="120" customHeight="1">
       <c r="A231" s="9" t="n">
@@ -14283,6 +14530,7 @@
         </is>
       </c>
       <c r="L231" s="9" t="inlineStr"/>
+      <c r="M231" s="9" t="inlineStr"/>
     </row>
     <row r="232" ht="120" customHeight="1">
       <c r="A232" s="7" t="n">
@@ -14339,6 +14587,7 @@
         </is>
       </c>
       <c r="L232" s="7" t="inlineStr"/>
+      <c r="M232" s="7" t="inlineStr"/>
     </row>
     <row r="233" ht="120" customHeight="1">
       <c r="A233" s="9" t="n">
@@ -14395,6 +14644,7 @@
         </is>
       </c>
       <c r="L233" s="9" t="inlineStr"/>
+      <c r="M233" s="9" t="inlineStr"/>
     </row>
     <row r="234" ht="120" customHeight="1">
       <c r="A234" s="7" t="n">
@@ -14451,6 +14701,7 @@
         </is>
       </c>
       <c r="L234" s="7" t="inlineStr"/>
+      <c r="M234" s="7" t="inlineStr"/>
     </row>
     <row r="235" ht="120" customHeight="1">
       <c r="A235" s="9" t="n">
@@ -14507,6 +14758,7 @@
         </is>
       </c>
       <c r="L235" s="9" t="inlineStr"/>
+      <c r="M235" s="9" t="inlineStr"/>
     </row>
     <row r="236" ht="120" customHeight="1">
       <c r="A236" s="7" t="n">
@@ -14563,6 +14815,7 @@
         </is>
       </c>
       <c r="L236" s="7" t="inlineStr"/>
+      <c r="M236" s="7" t="inlineStr"/>
     </row>
     <row r="237" ht="120" customHeight="1">
       <c r="A237" s="9" t="n">
@@ -14619,6 +14872,7 @@
         </is>
       </c>
       <c r="L237" s="9" t="inlineStr"/>
+      <c r="M237" s="9" t="inlineStr"/>
     </row>
     <row r="238" ht="120" customHeight="1">
       <c r="A238" s="7" t="n">
@@ -14675,6 +14929,7 @@
         </is>
       </c>
       <c r="L238" s="7" t="inlineStr"/>
+      <c r="M238" s="7" t="inlineStr"/>
     </row>
     <row r="239" ht="120" customHeight="1">
       <c r="A239" s="9" t="n">
@@ -14731,6 +14986,7 @@
         </is>
       </c>
       <c r="L239" s="9" t="inlineStr"/>
+      <c r="M239" s="9" t="inlineStr"/>
     </row>
     <row r="240" ht="120" customHeight="1">
       <c r="A240" s="7" t="n">
@@ -14787,6 +15043,7 @@
         </is>
       </c>
       <c r="L240" s="7" t="inlineStr"/>
+      <c r="M240" s="7" t="inlineStr"/>
     </row>
     <row r="241" ht="120" customHeight="1">
       <c r="A241" s="9" t="n">
@@ -14843,6 +15100,7 @@
         </is>
       </c>
       <c r="L241" s="9" t="inlineStr"/>
+      <c r="M241" s="9" t="inlineStr"/>
     </row>
     <row r="242" ht="120" customHeight="1">
       <c r="A242" s="7" t="n">
@@ -14899,6 +15157,7 @@
         </is>
       </c>
       <c r="L242" s="7" t="inlineStr"/>
+      <c r="M242" s="7" t="inlineStr"/>
     </row>
     <row r="243" ht="120" customHeight="1">
       <c r="A243" s="9" t="n">
@@ -14936,17 +15195,17 @@
       </c>
       <c r="H243" s="9" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I243" s="9" t="inlineStr">
         <is>
-          <t>a round button symbol of an upward arrow, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of an upward arrow, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J243" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K243" s="9" t="inlineStr">
@@ -14955,6 +15214,7 @@
         </is>
       </c>
       <c r="L243" s="9" t="inlineStr"/>
+      <c r="M243" s="9" t="inlineStr"/>
     </row>
     <row r="244" ht="120" customHeight="1">
       <c r="A244" s="7" t="n">
@@ -14992,17 +15252,17 @@
       </c>
       <c r="H244" s="7" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I244" s="7" t="inlineStr">
         <is>
-          <t>a round button symbol of a raised hand asking for help, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a raised hand asking for help, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J244" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K244" s="7" t="inlineStr">
@@ -15011,6 +15271,7 @@
         </is>
       </c>
       <c r="L244" s="7" t="inlineStr"/>
+      <c r="M244" s="7" t="inlineStr"/>
     </row>
     <row r="245" ht="120" customHeight="1">
       <c r="A245" s="9" t="n">
@@ -15048,17 +15309,17 @@
       </c>
       <c r="H245" s="9" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I245" s="9" t="inlineStr">
         <is>
-          <t>a round button symbol of two crossing kite strings, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of two crossing kite strings, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J245" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K245" s="9" t="inlineStr">
@@ -15067,6 +15328,7 @@
         </is>
       </c>
       <c r="L245" s="9" t="inlineStr"/>
+      <c r="M245" s="9" t="inlineStr"/>
     </row>
     <row r="246" ht="120" customHeight="1">
       <c r="A246" s="7" t="n">
@@ -15104,17 +15366,17 @@
       </c>
       <c r="H246" s="7" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I246" s="7" t="inlineStr">
         <is>
-          <t>a round button symbol of a small shield with a kite, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a small shield with a kite, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J246" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K246" s="7" t="inlineStr">
@@ -15123,6 +15385,7 @@
         </is>
       </c>
       <c r="L246" s="7" t="inlineStr"/>
+      <c r="M246" s="7" t="inlineStr"/>
     </row>
     <row r="247" ht="120" customHeight="1">
       <c r="A247" s="9" t="n">
@@ -15160,17 +15423,17 @@
       </c>
       <c r="H247" s="9" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I247" s="9" t="inlineStr">
         <is>
-          <t>a round button symbol of a wooden crate, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a wooden crate, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J247" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K247" s="9" t="inlineStr">
@@ -15179,6 +15442,7 @@
         </is>
       </c>
       <c r="L247" s="9" t="inlineStr"/>
+      <c r="M247" s="9" t="inlineStr"/>
     </row>
     <row r="248" ht="120" customHeight="1">
       <c r="A248" s="7" t="n">
@@ -15216,17 +15480,17 @@
       </c>
       <c r="H248" s="7" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I248" s="7" t="inlineStr">
         <is>
-          <t>a round button symbol of a cut thread with a spark, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a cut thread with a spark, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J248" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K248" s="7" t="inlineStr">
@@ -15235,6 +15499,7 @@
         </is>
       </c>
       <c r="L248" s="7" t="inlineStr"/>
+      <c r="M248" s="7" t="inlineStr"/>
     </row>
     <row r="249" ht="120" customHeight="1">
       <c r="A249" s="9" t="n">
@@ -15272,17 +15537,17 @@
       </c>
       <c r="H249" s="9" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I249" s="9" t="inlineStr">
         <is>
-          <t>a round button symbol of a hand on heart, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of a hand on heart, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J249" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K249" s="9" t="inlineStr">
@@ -15291,6 +15556,7 @@
         </is>
       </c>
       <c r="L249" s="9" t="inlineStr"/>
+      <c r="M249" s="9" t="inlineStr"/>
     </row>
     <row r="250" ht="120" customHeight="1">
       <c r="A250" s="7" t="n">
@@ -15328,17 +15594,17 @@
       </c>
       <c r="H250" s="7" t="inlineStr">
         <is>
-          <t>Flat painted symbol inside a circle. Readable at 48 px.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Readable at 48 px.</t>
         </is>
       </c>
       <c r="I250" s="7" t="inlineStr">
         <is>
-          <t>a round button symbol of two hands shaking, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple flat white silhouette symbol of two hands shaking, pure white on transparent background, clean edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J250" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K250" s="7" t="inlineStr">
@@ -15347,6 +15613,7 @@
         </is>
       </c>
       <c r="L250" s="7" t="inlineStr"/>
+      <c r="M250" s="7" t="inlineStr"/>
     </row>
     <row r="251" ht="120" customHeight="1">
       <c r="A251" s="9" t="n">
@@ -15384,17 +15651,17 @@
       </c>
       <c r="H251" s="9" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I251" s="9" t="inlineStr">
         <is>
-          <t>a bold simple icon of an unwinding spool with thread flowing out (release), single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of an unwinding spool with thread flowing out (release), pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J251" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K251" s="9" t="inlineStr">
@@ -15403,6 +15670,7 @@
         </is>
       </c>
       <c r="L251" s="9" t="inlineStr"/>
+      <c r="M251" s="9" t="inlineStr"/>
     </row>
     <row r="252" ht="120" customHeight="1">
       <c r="A252" s="7" t="n">
@@ -15440,17 +15708,17 @@
       </c>
       <c r="H252" s="7" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I252" s="7" t="inlineStr">
         <is>
-          <t>a bold simple icon of a hand pulling thread back hard (pull), single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a hand pulling thread back hard (pull), pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J252" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K252" s="7" t="inlineStr">
@@ -15459,6 +15727,7 @@
         </is>
       </c>
       <c r="L252" s="7" t="inlineStr"/>
+      <c r="M252" s="7" t="inlineStr"/>
     </row>
     <row r="253" ht="120" customHeight="1">
       <c r="A253" s="9" t="n">
@@ -15496,17 +15765,17 @@
       </c>
       <c r="H253" s="9" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I253" s="9" t="inlineStr">
         <is>
-          <t>a bold simple icon of a vintage microphone, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a vintage microphone, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J253" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K253" s="9" t="inlineStr">
@@ -15515,6 +15784,7 @@
         </is>
       </c>
       <c r="L253" s="9" t="inlineStr"/>
+      <c r="M253" s="9" t="inlineStr"/>
     </row>
     <row r="254" ht="120" customHeight="1">
       <c r="A254" s="7" t="n">
@@ -15552,17 +15822,17 @@
       </c>
       <c r="H254" s="7" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I254" s="7" t="inlineStr">
         <is>
-          <t>a bold simple icon of a vintage speaker horn, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a vintage speaker horn, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J254" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K254" s="7" t="inlineStr">
@@ -15571,6 +15841,7 @@
         </is>
       </c>
       <c r="L254" s="7" t="inlineStr"/>
+      <c r="M254" s="7" t="inlineStr"/>
     </row>
     <row r="255" ht="120" customHeight="1">
       <c r="A255" s="9" t="n">
@@ -15608,17 +15879,17 @@
       </c>
       <c r="H255" s="9" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I255" s="9" t="inlineStr">
         <is>
-          <t>a bold simple icon of a folded old paper map, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a folded old paper map, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J255" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K255" s="9" t="inlineStr">
@@ -15627,6 +15898,7 @@
         </is>
       </c>
       <c r="L255" s="9" t="inlineStr"/>
+      <c r="M255" s="9" t="inlineStr"/>
     </row>
     <row r="256" ht="120" customHeight="1">
       <c r="A256" s="7" t="n">
@@ -15664,17 +15936,17 @@
       </c>
       <c r="H256" s="7" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I256" s="7" t="inlineStr">
         <is>
-          <t>a bold simple icon of a kite folded under an arm, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a kite folded under an arm, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J256" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K256" s="7" t="inlineStr">
@@ -15683,6 +15955,7 @@
         </is>
       </c>
       <c r="L256" s="7" t="inlineStr"/>
+      <c r="M256" s="7" t="inlineStr"/>
     </row>
     <row r="257" ht="120" customHeight="1">
       <c r="A257" s="9" t="n">
@@ -15720,17 +15993,17 @@
       </c>
       <c r="H257" s="9" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I257" s="9" t="inlineStr">
         <is>
-          <t>a bold simple icon of a kite rising from a hand, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a kite rising from a hand, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J257" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K257" s="9" t="inlineStr">
@@ -15739,6 +16012,7 @@
         </is>
       </c>
       <c r="L257" s="9" t="inlineStr"/>
+      <c r="M257" s="9" t="inlineStr"/>
     </row>
     <row r="258" ht="120" customHeight="1">
       <c r="A258" s="7" t="n">
@@ -15776,17 +16050,17 @@
       </c>
       <c r="H258" s="7" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I258" s="7" t="inlineStr">
         <is>
-          <t>a bold simple icon of wind swirl lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of wind swirl lines, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J258" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K258" s="7" t="inlineStr">
@@ -15795,6 +16069,7 @@
         </is>
       </c>
       <c r="L258" s="7" t="inlineStr"/>
+      <c r="M258" s="7" t="inlineStr"/>
     </row>
     <row r="259" ht="120" customHeight="1">
       <c r="A259" s="9" t="n">
@@ -15832,17 +16107,17 @@
       </c>
       <c r="H259" s="9" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I259" s="9" t="inlineStr">
         <is>
-          <t>a bold simple icon of a straining thread about to snap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a straining thread about to snap, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J259" s="9" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K259" s="9" t="inlineStr">
@@ -15851,6 +16126,7 @@
         </is>
       </c>
       <c r="L259" s="9" t="inlineStr"/>
+      <c r="M259" s="9" t="inlineStr"/>
     </row>
     <row r="260" ht="120" customHeight="1">
       <c r="A260" s="7" t="n">
@@ -15888,17 +16164,17 @@
       </c>
       <c r="H260" s="7" t="inlineStr">
         <is>
-          <t>UI button glyph. Designer may simplify to flat 2-colour for clarity. Thumb-size buttons.</t>
+          <t>WHITE glyph on transparent background (the game tints it). Simple bold shape, thumb-size button.</t>
         </is>
       </c>
       <c r="I260" s="7" t="inlineStr">
         <is>
-          <t>a bold simple icon of a smiling face, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bold simple flat white silhouette icon of a smiling face, pure white on transparent background, clean vector-like edges, no shading, game UI glyph</t>
         </is>
       </c>
       <c r="J260" s="7" t="inlineStr">
         <is>
-          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box</t>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
         </is>
       </c>
       <c r="K260" s="7" t="inlineStr">
@@ -15907,6 +16183,7 @@
         </is>
       </c>
       <c r="L260" s="7" t="inlineStr"/>
+      <c r="M260" s="7" t="inlineStr"/>
     </row>
     <row r="261" ht="120" customHeight="1">
       <c r="A261" s="9" t="n">
@@ -15963,6 +16240,7 @@
         </is>
       </c>
       <c r="L261" s="9" t="inlineStr"/>
+      <c r="M261" s="9" t="inlineStr"/>
     </row>
     <row r="262" ht="120" customHeight="1">
       <c r="A262" s="7" t="n">
@@ -16019,6 +16297,7 @@
         </is>
       </c>
       <c r="L262" s="7" t="inlineStr"/>
+      <c r="M262" s="7" t="inlineStr"/>
     </row>
     <row r="263" ht="120" customHeight="1">
       <c r="A263" s="9" t="n">
@@ -16075,6 +16354,7 @@
         </is>
       </c>
       <c r="L263" s="9" t="inlineStr"/>
+      <c r="M263" s="9" t="inlineStr"/>
     </row>
     <row r="264" ht="120" customHeight="1">
       <c r="A264" s="7" t="n">
@@ -16131,6 +16411,7 @@
         </is>
       </c>
       <c r="L264" s="7" t="inlineStr"/>
+      <c r="M264" s="7" t="inlineStr"/>
     </row>
     <row r="265" ht="120" customHeight="1">
       <c r="A265" s="9" t="n">
@@ -16187,6 +16468,7 @@
         </is>
       </c>
       <c r="L265" s="9" t="inlineStr"/>
+      <c r="M265" s="9" t="inlineStr"/>
     </row>
     <row r="266" ht="120" customHeight="1">
       <c r="A266" s="7" t="n">
@@ -16243,6 +16525,7 @@
         </is>
       </c>
       <c r="L266" s="7" t="inlineStr"/>
+      <c r="M266" s="7" t="inlineStr"/>
     </row>
     <row r="267" ht="120" customHeight="1">
       <c r="A267" s="9" t="n">
@@ -16299,6 +16582,7 @@
         </is>
       </c>
       <c r="L267" s="9" t="inlineStr"/>
+      <c r="M267" s="9" t="inlineStr"/>
     </row>
     <row r="268" ht="120" customHeight="1">
       <c r="A268" s="7" t="n">
@@ -16355,6 +16639,7 @@
         </is>
       </c>
       <c r="L268" s="7" t="inlineStr"/>
+      <c r="M268" s="7" t="inlineStr"/>
     </row>
     <row r="269" ht="120" customHeight="1">
       <c r="A269" s="9" t="n">
@@ -16411,6 +16696,7 @@
         </is>
       </c>
       <c r="L269" s="9" t="inlineStr"/>
+      <c r="M269" s="9" t="inlineStr"/>
     </row>
     <row r="270" ht="120" customHeight="1">
       <c r="A270" s="7" t="n">
@@ -16467,6 +16753,7 @@
         </is>
       </c>
       <c r="L270" s="7" t="inlineStr"/>
+      <c r="M270" s="7" t="inlineStr"/>
     </row>
     <row r="271" ht="120" customHeight="1">
       <c r="A271" s="9" t="n">
@@ -16523,6 +16810,7 @@
         </is>
       </c>
       <c r="L271" s="9" t="inlineStr"/>
+      <c r="M271" s="9" t="inlineStr"/>
     </row>
     <row r="272" ht="120" customHeight="1">
       <c r="A272" s="7" t="n">
@@ -16579,6 +16867,7 @@
         </is>
       </c>
       <c r="L272" s="7" t="inlineStr"/>
+      <c r="M272" s="7" t="inlineStr"/>
     </row>
     <row r="273" ht="120" customHeight="1">
       <c r="A273" s="9" t="n">
@@ -16635,6 +16924,7 @@
         </is>
       </c>
       <c r="L273" s="9" t="inlineStr"/>
+      <c r="M273" s="9" t="inlineStr"/>
     </row>
     <row r="274" ht="120" customHeight="1">
       <c r="A274" s="7" t="n">
@@ -16691,6 +16981,7 @@
         </is>
       </c>
       <c r="L274" s="7" t="inlineStr"/>
+      <c r="M274" s="7" t="inlineStr"/>
     </row>
     <row r="275" ht="120" customHeight="1">
       <c r="A275" s="9" t="n">
@@ -16747,6 +17038,7 @@
         </is>
       </c>
       <c r="L275" s="9" t="inlineStr"/>
+      <c r="M275" s="9" t="inlineStr"/>
     </row>
     <row r="276" ht="120" customHeight="1">
       <c r="A276" s="7" t="n">
@@ -16803,6 +17095,7 @@
         </is>
       </c>
       <c r="L276" s="7" t="inlineStr"/>
+      <c r="M276" s="7" t="inlineStr"/>
     </row>
     <row r="277" ht="120" customHeight="1">
       <c r="A277" s="9" t="n">
@@ -16859,6 +17152,7 @@
         </is>
       </c>
       <c r="L277" s="9" t="inlineStr"/>
+      <c r="M277" s="9" t="inlineStr"/>
     </row>
     <row r="278" ht="120" customHeight="1">
       <c r="A278" s="7" t="n">
@@ -16915,6 +17209,7 @@
         </is>
       </c>
       <c r="L278" s="7" t="inlineStr"/>
+      <c r="M278" s="7" t="inlineStr"/>
     </row>
     <row r="279" ht="120" customHeight="1">
       <c r="A279" s="9" t="n">
@@ -16971,9 +17266,10 @@
         </is>
       </c>
       <c r="L279" s="9" t="inlineStr"/>
+      <c r="M279" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L279"/>
+  <autoFilter ref="A1:M279"/>
   <dataValidations count="1">
     <dataValidation sqref="K2:K279" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,In progress,Review,Approved,In Unity"</formula1>

</xml_diff>

<commit_message>
Make Kitefall international: project rules, global art style, plan
CLAUDE.md records the project rules (international audience first, safety,
fair play). Decision D57 and docs/INTERNATIONAL_PLAN.md list what changes for
a worldwide audience: English-first UI words, languages, kites/arenas/
characters from other kite cultures, events, store and privacy. The image
prompts now use a classical storybook world-festival style. Image Mapper can
export the list of images still missing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kft94361aqxz3Q9WMshigR
</commit_message>
<xml_diff>
--- a/docs/Kitefall_Image_Assets.xlsx
+++ b/docs/Kitefall_Image_Assets.xlsx
@@ -522,7 +522,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Art direction</t>
@@ -530,11 +530,11 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Classical South Asian miniature painting + premium mobile game polish. Hand-painted gouache feel, fine gold-leaf ornament, warm golden-hour light. Elegant, festive, friendly – never dark or violent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
+          <t>INTERNATIONAL game: classical hand-painted storybook look that welcomes players worldwide + premium mobile polish. Gouache feel, fine gold ornament, warm golden-hour light. Regional items (an arena, a character, a kite) may show their own culture respectfully; menus, branding and UI stay globally neutral. Elegant, festive, friendly – never dark or violent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Master style prompt (add to every prompt)</t>
@@ -542,7 +542,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>A single majestic diamond-shaped paper kite in saffron and vermilion with an ornate gold-leaf mandala pattern, soaring against a glowing sunset sky, flowing ribbon tail curling around it, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design, bold simple icon composition, high contrast</t>
+          <t>A single majestic diamond-shaped paper kite in saffron and vermilion with an ornate gold-leaf mandala pattern, soaring against a glowing sunset sky, flowing ribbon tail curling around it, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design, bold simple icon composition, high contrast</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>The same ornate saffron and vermilion diamond paper kite with curling ribbon tail, centred, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>The same ornate saffron and vermilion diamond paper kite with curling ribbon tail, centred, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Soft warm sunset sky gradient from deep indigo to saffron with very faint gold-leaf geometric jali pattern, seamless, no objects, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Soft warm sunset sky gradient from deep indigo to saffron with very faint gold-leaf geometric jali pattern, seamless, no objects, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>Ornamental title cartouche emblem with empty centre space for a word, gold-leaf arabesque scrollwork, a small paper kite and ribbon flourish on the left, symmetrical, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Ornamental title cartouche emblem with empty centre space for a word, gold-leaf arabesque scrollwork, a small paper kite and ribbon flourish on the left, symmetrical, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Breathtaking panoramic view of an old walled city at golden hour, dense stacked brick rooftops with carved wooden balconies, hundreds of colourful paper kites filling the sky, a young flyer silhouetted on a rooftop holding a wooden spool, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Breathtaking panoramic view of an old walled city at golden hour, dense stacked brick rooftops with carved wooden balconies, hundreds of colourful paper kites filling the sky, a young flyer silhouetted on a rooftop holding a wooden spool, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>children and families on old city rooftops at sunrise preparing kites, marigold garlands and string lights, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>children and families on old city rooftops at sunrise preparing kites, marigold garlands and string lights, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>seaside cliff houses painted white and teal, kites flying over a turquoise sea with fishing boats, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>seaside cliff houses painted white and teal, kites flying over a turquoise sea with fishing boats, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>a riverside spring festival with lantern boats, temple steps and kites reflected in calm water, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a riverside spring festival with lantern boats, temple steps and kites reflected in calm water, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>a grand palace garden with marble pavilions, fountains and royal kite flyers on terraces, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a grand palace garden with marble pavilions, fountains and royal kite flyers on terraces, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>a terraced mountain village with prayer-flag-like coloured cloth and kites over snowy peaks, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a terraced mountain village with prayer-flag-like coloured cloth and kites over snowy peaks, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>an island archipelago under dramatic storm clouds with brave kites cutting through the wind, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an island archipelago under dramatic storm clouds with brave kites cutting through the wind, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Two ornate paper kites, one saffron and one indigo, crossing strings dramatically in a glowing festival sky above old city rooftops, sense of a friendly rooftop duel, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Two ornate paper kites, one saffron and one indigo, crossing strings dramatically in a glowing festival sky above old city rooftops, sense of a friendly rooftop duel, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Decorative landscape banner frame with an empty centre window, gold-leaf border with floral arabesques and tiny kites in the corners, deep indigo velvet background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>a cosy rooftop at golden hour with a charpai bed, potted plants, wooden spools and a kite rack, city of rooftops behind, kites in the sky, gentle and inviting, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a cosy rooftop at golden hour with a wooden day-bed, potted plants, wooden spools and a kite rack, city of rooftops behind, kites in the sky, gentle and inviting, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>an old bazaar kite stall with kites hanging from wooden beams, spools of coloured cotton thread on shelves, warm lantern light, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an old bazaar kite stall with kites hanging from wooden beams, spools of coloured cotton thread on shelves, warm lantern light, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>a craftsman's kite workshop with bamboo sticks, tissue paper sheets, glue pots, painted wooden spools, soft window light, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a craftsman's kite workshop with bamboo sticks, tissue paper sheets, glue pots, painted wooden spools, soft window light, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>an elegant tailor's room with folded festive clothes, carved wooden mirror frame, embroidered curtains, a soft spotlight circle on the floor in the centre, cinematic composition, soft depth of field, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an elegant tailor's room with folded festive clothes, carved wooden mirror frame, embroidered curtains, a soft spotlight circle on the floor in the centre, cinematic composition, soft depth of field, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>a wide rooftop terrace at dusk with four empty spots marked by rugs for friends to stand, string lights overhead, cinematic composition, soft depth of field, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wide rooftop terrace at dusk with four empty spots marked by rugs for friends to stand, string lights overhead, cinematic composition, soft depth of field, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>a grand festive night sky with fireworks-like lantern lights, golden kites rising in a spiral, royal ornamental feel, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a grand festive night sky with fireworks-like lantern lights, golden kites rising in a spiral, royal ornamental feel, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>a triumphant golden sunrise sky with confetti of paper petals and a single proud kite rising high, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a triumphant golden sunrise sky with confetti of paper petals and a single proud kite rising high, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>a calm twilight sky with a lone kite drifting gently down, peaceful and hopeful, not sad, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a calm twilight sky with a lone kite drifting gently down, peaceful and hopeful, not sad, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>a soft blurred rooftop evening with very low detail, subtle gold pattern, calm, cinematic composition, soft depth of field, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a soft blurred rooftop evening with very low detail, subtle gold pattern, calm, cinematic composition, soft depth of field, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>An elegant classic South Asian diamond fighter kite (guddi/patang) with a curved bamboo spine and bow, small triangular tail flap, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant classic South Asian diamond fighter kite (guddi/patang) with a curved bamboo spine and bow, small triangular tail flap, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>An elegant small square fighter kite (pipa) with a central bamboo spine and arched cross-bow, light and nimble, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant small square fighter kite (pipa) with a central bamboo spine and arched cross-bow, light and nimble, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I33" s="9" t="inlineStr">
         <is>
-          <t>An elegant six-sided tall hexagonal kite (rokkaku style) with two cross spars, bold painted panels, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant six-sided tall hexagonal kite (rokkaku style) with two cross spars, bold painted panels, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>An elegant small Thai-style diamond fighter kite (pakpao) with long thin tail strings, agile shape, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant small Thai-style diamond fighter kite (pakpao) with long thin tail strings, agile shape, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="I35" s="9" t="inlineStr">
         <is>
-          <t>An elegant Afghan-style fighter kite (gudiparan) with a wide diamond body and a tiny tassel tail, elegant curved bow, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant Afghan-style fighter kite (gudiparan) with a wide diamond body and a tiny tassel tail, elegant curved bow, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J35" s="9" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>An elegant large Thai star-shaped kite (chula) with five pointed bamboo arms, powerful and grand, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant large Thai star-shaped kite (chula) with five pointed bamboo arms, powerful and grand, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="I37" s="9" t="inlineStr">
         <is>
-          <t>An elegant Malaysian moon kite (wau bulan) with a crescent tail, wide curved wings and intricate floral cut-paper decoration, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>An elegant Malaysian moon kite (wau bulan) with a crescent tail, wide curved wings and intricate floral cut-paper decoration, made of translucent tissue paper on bamboo sticks, ivory and gold base colours with subtle hand-painted border lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J37" s="9" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="I39" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, royal blue and pale sky blue colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, royal blue and pale sky blue colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J39" s="9" t="inlineStr">
@@ -3629,7 +3629,7 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, deep violet and rose pink colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, deep violet and rose pink colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, teal and mint white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, teal and mint white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J42" s="7" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="I43" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, saffron orange and pure white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, saffron orange and pure white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J43" s="9" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, jade green and soft lime colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, jade green and soft lime colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J44" s="7" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="I45" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a guddi kite sail as a design sheet, deep crimson and charcoal black colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a guddi kite sail as a design sheet, deep crimson and charcoal black colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J45" s="9" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J46" s="7" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="I47" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, royal blue and pale sky blue colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, royal blue and pale sky blue colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J47" s="9" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="I49" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, deep violet and rose pink colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, deep violet and rose pink colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J49" s="9" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="I50" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, teal and mint white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, teal and mint white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J50" s="7" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="I51" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, saffron orange and pure white colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, saffron orange and pure white colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J51" s="9" t="inlineStr">
@@ -4313,7 +4313,7 @@
       </c>
       <c r="I52" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, jade green and soft lime colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, jade green and soft lime colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J52" s="7" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="I53" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pipa kite sail as a design sheet, deep crimson and charcoal black colour scheme, sunburst rays hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pipa kite sail as a design sheet, deep crimson and charcoal black colour scheme, sunburst rays hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J53" s="9" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J54" s="7" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="I55" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, royal blue and pale sky blue colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, royal blue and pale sky blue colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J55" s="9" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="I57" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, deep violet and rose pink colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, deep violet and rose pink colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J57" s="9" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="I58" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, teal and mint white colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, teal and mint white colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J58" s="7" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, saffron orange and pure white colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, saffron orange and pure white colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J59" s="9" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="I60" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, jade green and soft lime colour scheme, sunburst rays hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, jade green and soft lime colour scheme, sunburst rays hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J60" s="7" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="I61" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, deep crimson and charcoal black colour scheme, paisley motifs hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a rokkaku kite sail as a design sheet, deep crimson and charcoal black colour scheme, paisley motifs hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J61" s="9" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J62" s="7" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="I63" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, royal blue and pale sky blue colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, royal blue and pale sky blue colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J63" s="9" t="inlineStr">
@@ -4997,7 +4997,7 @@
       </c>
       <c r="I64" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J64" s="7" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="I65" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, deep violet and rose pink colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, deep violet and rose pink colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J65" s="9" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, teal and mint white colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, teal and mint white colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J66" s="7" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="I67" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, saffron orange and pure white colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, saffron orange and pure white colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J67" s="9" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="I68" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, jade green and soft lime colour scheme, paisley motifs hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, jade green and soft lime colour scheme, paisley motifs hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J68" s="7" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="I69" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, deep crimson and charcoal black colour scheme, lotus mandala hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a pakpao kite sail as a design sheet, deep crimson and charcoal black colour scheme, lotus mandala hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J69" s="9" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J70" s="7" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="I71" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, royal blue and pale sky blue colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, royal blue and pale sky blue colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="I72" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J72" s="7" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, deep violet and rose pink colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, deep violet and rose pink colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J73" s="9" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, teal and mint white colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, teal and mint white colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J74" s="7" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="I75" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, saffron orange and pure white colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, saffron orange and pure white colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J75" s="9" t="inlineStr">
@@ -5681,7 +5681,7 @@
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, jade green and soft lime colour scheme, lotus mandala hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, jade green and soft lime colour scheme, lotus mandala hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J76" s="7" t="inlineStr">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="I77" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, deep crimson and charcoal black colour scheme, block-print stripes hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a gudiparan kite sail as a design sheet, deep crimson and charcoal black colour scheme, block-print stripes hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J77" s="9" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J78" s="7" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="I79" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, royal blue and pale sky blue colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, royal blue and pale sky blue colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J79" s="9" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J80" s="7" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="I81" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, deep violet and rose pink colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, deep violet and rose pink colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr">
@@ -6023,7 +6023,7 @@
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, teal and mint white colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, teal and mint white colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J82" s="7" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="I83" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, saffron orange and pure white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, saffron orange and pure white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J83" s="9" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="I84" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, jade green and soft lime colour scheme, block-print stripes hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, jade green and soft lime colour scheme, block-print stripes hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J84" s="7" t="inlineStr">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="I85" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a chula kite sail as a design sheet, deep crimson and charcoal black colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a chula kite sail as a design sheet, deep crimson and charcoal black colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J85" s="9" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="I86" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, vermilion red and warm butter yellow colour scheme, Mughal floral border hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J86" s="7" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="I87" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, royal blue and pale sky blue colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, royal blue and pale sky blue colour scheme, geometric jali lattice hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J87" s="9" t="inlineStr">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="I88" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, mustard yellow and fresh leaf green colour scheme, sunburst rays hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J88" s="7" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="I89" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, deep violet and rose pink colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, deep violet and rose pink colour scheme, paisley motifs hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J89" s="9" t="inlineStr">
@@ -6479,7 +6479,7 @@
       </c>
       <c r="I90" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, teal and mint white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, teal and mint white colour scheme, lotus mandala hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J90" s="7" t="inlineStr">
@@ -6536,7 +6536,7 @@
       </c>
       <c r="I91" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, saffron orange and pure white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, saffron orange and pure white colour scheme, block-print stripes hand-painted on thin tissue paper, fine ink linework, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J91" s="9" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="I92" s="7" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, jade green and soft lime colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, jade green and soft lime colour scheme, Mughal floral border hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J92" s="7" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="I93" s="9" t="inlineStr">
         <is>
-          <t>Flat front-on artwork of a wau kite sail as a design sheet, deep crimson and charcoal black colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Flat front-on artwork of a wau kite sail as a design sheet, deep crimson and charcoal black colour scheme, geometric jali lattice hand-painted on thin tissue paper, rich gold-leaf ornament, symmetrical, fills the frame edge to edge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J93" s="9" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="I94" s="7" t="inlineStr">
         <is>
-          <t>an empty dashed circle meaning no tail, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an empty dashed circle meaning no tail, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J94" s="7" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="I95" s="9" t="inlineStr">
         <is>
-          <t>a short single silk-like ribbon tail curling in the wind, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a short single silk-like ribbon tail curling in the wind, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J95" s="9" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="I96" s="7" t="inlineStr">
         <is>
-          <t>two parallel ribbon tails fluttering, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>two parallel ribbon tails fluttering, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J96" s="7" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="I97" s="9" t="inlineStr">
         <is>
-          <t>a very long flowing cloth tail with small bows, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a very long flowing cloth tail with small bows, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J97" s="9" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="I98" s="7" t="inlineStr">
         <is>
-          <t>a decorative cotton tassel with tiny beads, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a decorative cotton tassel with tiny beads, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J98" s="7" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="I99" s="9" t="inlineStr">
         <is>
-          <t>a hand-wound ball of plain natural cotton thread, honest and simple, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a hand-wound ball of plain natural cotton thread, honest and simple, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J99" s="9" t="inlineStr">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="I100" s="7" t="inlineStr">
         <is>
-          <t>a smooth lustrous ball of fine silk-like thread with soft sheen, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a smooth lustrous ball of fine silk-like thread with soft sheen, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J100" s="7" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="I101" s="9" t="inlineStr">
         <is>
-          <t>a tightly wound ball of thick deep-crimson dyed cotton thread with a bold aggressive look, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a tightly wound ball of thick deep-crimson dyed cotton thread with a bold aggressive look, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J101" s="9" t="inlineStr">
@@ -7163,7 +7163,7 @@
       </c>
       <c r="I102" s="7" t="inlineStr">
         <is>
-          <t>a heavy thick braided cotton cord wound in a ball, sturdy and strong, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heavy thick braided cotton cord wound in a ball, sturdy and strong, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J102" s="7" t="inlineStr">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="I103" s="9" t="inlineStr">
         <is>
-          <t>a very large ball of long thin cotton thread, generous and abundant, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a very large ball of long thin cotton thread, generous and abundant, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J103" s="9" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="I104" s="7" t="inlineStr">
         <is>
-          <t>a springy loosely coiled ball of soft flexible cotton thread, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a springy loosely coiled ball of soft flexible cotton thread, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J104" s="7" t="inlineStr">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="I105" s="9" t="inlineStr">
         <is>
-          <t>a classic carved wooden kite spool (charkhi) with two handles, warm walnut wood, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a classic carved wooden kite spool (charkhi) with two handles, warm walnut wood, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J105" s="9" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="I106" s="7" t="inlineStr">
         <is>
-          <t>a slim lightweight wooden kite spool with streamlined spokes and red lacquer stripes, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a slim lightweight wooden kite spool with streamlined spokes and red lacquer stripes, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J106" s="7" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="I107" s="9" t="inlineStr">
         <is>
-          <t>a large wide-drum wooden kite spool holding lots of thread, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a large wide-drum wooden kite spool holding lots of thread, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J107" s="9" t="inlineStr">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="I108" s="7" t="inlineStr">
         <is>
-          <t>a sturdy wooden kite spool with a leather friction strap wrapped around one handle, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a sturdy wooden kite spool with a leather friction strap wrapped around one handle, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J108" s="7" t="inlineStr">
@@ -7562,7 +7562,7 @@
       </c>
       <c r="I109" s="9" t="inlineStr">
         <is>
-          <t>an ornate wooden kite spool with carved cog-like rims and brass-coloured painted details, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an ornate wooden kite spool with carved cog-like rims and brass-coloured painted details, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J109" s="9" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="I110" s="7" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing a small pot of beeswax with a cotton thread passing over it, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing a small pot of beeswax with a cotton thread passing over it, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J110" s="7" t="inlineStr">
@@ -7676,7 +7676,7 @@
       </c>
       <c r="I111" s="9" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing two cotton threads twisting together into one, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing two cotton threads twisting together into one, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J111" s="9" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="I112" s="7" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing a feather-light wisp of thread floating upward, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing a feather-light wisp of thread floating upward, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J112" s="7" t="inlineStr">
@@ -7790,7 +7790,7 @@
       </c>
       <c r="I113" s="9" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing a tiny oil can dripping one drop onto a wooden axle, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing a tiny oil can dripping one drop onto a wooden axle, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J113" s="9" t="inlineStr">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="I114" s="7" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing a wide wooden drum spool seen from the side, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing a wide wooden drum spool seen from the side, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J114" s="7" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="I115" s="9" t="inlineStr">
         <is>
-          <t>a round ornate gold medallion badge containing a soft wrapped cloth handle grip, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate gold medallion badge containing a soft wrapped cloth handle grip, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J115" s="9" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="I116" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Ali, a cheerful young man from an old South Asian city, short dark hair, warm brown skin, street kurta, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Ali, a cheerful young man from an old South Asian city, short dark hair, warm brown skin, street kurta, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J116" s="7" t="inlineStr">
@@ -8018,7 +8018,7 @@
       </c>
       <c r="I117" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Ali, a cheerful young man from an old South Asian city, short dark hair, warm brown skin, street kurta, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Ali, a cheerful young man from an old South Asian city, short dark hair, warm brown skin, street kurta, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J117" s="9" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="I118" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Sana, a confident young woman with long braided dark hair, light brown skin, bright yellow and green festive outfit, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Sana, a confident young woman with long braided dark hair, light brown skin, bright yellow and green festive outfit, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J118" s="7" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="I119" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Sana, a confident young woman with long braided dark hair, light brown skin, bright yellow and green festive outfit, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Sana, a confident young woman with long braided dark hair, light brown skin, bright yellow and green festive outfit, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J119" s="9" t="inlineStr">
@@ -8189,7 +8189,7 @@
       </c>
       <c r="I120" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Zara, a stylish young woman from Lahore with a high bun, deep violet and orange night-bazaar outfit, playful smile, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Zara, a stylish young woman from Lahore with a high bun, deep violet and orange night-bazaar outfit, playful smile, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J120" s="7" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="I121" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Zara, a stylish young woman from Lahore with a high bun, deep violet and orange night-bazaar outfit, playful smile, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Zara, a stylish young woman from Lahore with a high bun, deep violet and orange night-bazaar outfit, playful smile, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J121" s="9" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="I122" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Rafay, a tall broad-shouldered young man from Karachi, buzz-cut hair, coastal linen shirt in white and teal, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Rafay, a tall broad-shouldered young man from Karachi, buzz-cut hair, coastal linen shirt in white and teal, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J122" s="7" t="inlineStr">
@@ -8360,7 +8360,7 @@
       </c>
       <c r="I123" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Rafay, a tall broad-shouldered young man from Karachi, buzz-cut hair, coastal linen shirt in white and teal, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Rafay, a tall broad-shouldered young man from Karachi, buzz-cut hair, coastal linen shirt in white and teal, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J123" s="9" t="inlineStr">
@@ -8417,7 +8417,7 @@
       </c>
       <c r="I124" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Lucas, a friendly young man from Lisbon with wavy chestnut hair, fair skin, blue monsoon rain jacket, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Lucas, a friendly young man from Lisbon with wavy chestnut hair, fair skin, blue monsoon rain jacket, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J124" s="7" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="I125" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Lucas, a friendly young man from Lisbon with wavy chestnut hair, fair skin, blue monsoon rain jacket, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Lucas, a friendly young man from Lisbon with wavy chestnut hair, fair skin, blue monsoon rain jacket, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J125" s="9" t="inlineStr">
@@ -8531,7 +8531,7 @@
       </c>
       <c r="I126" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Aiko, an energetic young woman from Osaka with a sleek black bob, pink and yellow festival-lights jacket, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Aiko, an energetic young woman from Osaka with a sleek black bob, pink and yellow festival-lights jacket, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J126" s="7" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="I127" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Aiko, an energetic young woman from Osaka with a sleek black bob, pink and yellow festival-lights jacket, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Aiko, an energetic young woman from Osaka with a sleek black bob, pink and yellow festival-lights jacket, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J127" s="9" t="inlineStr">
@@ -8645,7 +8645,7 @@
       </c>
       <c r="I128" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Niran, a calm young man from Chiang Mai with short black hair, navy rooftop hoodie with orange trim, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Niran, a calm young man from Chiang Mai with short black hair, navy rooftop hoodie with orange trim, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J128" s="7" t="inlineStr">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="I129" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Niran, a calm young man from Chiang Mai with short black hair, navy rooftop hoodie with orange trim, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Niran, a calm young man from Chiang Mai with short black hair, navy rooftop hoodie with orange trim, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J129" s="9" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="I130" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Farid, a rugged young man from Kabul with tousled dark hair and short beard, red mountain parka, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Farid, a rugged young man from Kabul with tousled dark hair and short beard, red mountain parka, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J130" s="7" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="I131" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Farid, a rugged young man from Kabul with tousled dark hair and short beard, red mountain parka, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Farid, a rugged young man from Kabul with tousled dark hair and short beard, red mountain parka, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J131" s="9" t="inlineStr">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="I132" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Siti, a quick athletic young woman from Kuala Lumpur with a long ponytail, green and lime storm-runner outfit, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Siti, a quick athletic young woman from Kuala Lumpur with a long ponytail, green and lime storm-runner outfit, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J132" s="7" t="inlineStr">
@@ -8930,7 +8930,7 @@
       </c>
       <c r="I133" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Siti, a quick athletic young woman from Kuala Lumpur with a long ponytail, green and lime storm-runner outfit, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Siti, a quick athletic young woman from Kuala Lumpur with a long ponytail, green and lime storm-runner outfit, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J133" s="9" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="I134" s="7" t="inlineStr">
         <is>
-          <t>Portrait of Arjun, a dignified young man from Ahmedabad with neat black hair, cream and gold royal sherwani, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Portrait of Arjun, a dignified young man from Ahmedabad with neat black hair, cream and gold royal sherwani, holding a small paper kite near the shoulder, warm smile, three-quarter view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J134" s="7" t="inlineStr">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="I135" s="9" t="inlineStr">
         <is>
-          <t>Full-body character art of Arjun, a dignified young man from Ahmedabad with neat black hair, cream and gold royal sherwani, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Full-body character art of Arjun, a dignified young man from Ahmedabad with neat black hair, cream and gold royal sherwani, standing proudly on tiptoe holding a carved wooden kite spool, kite string rising out of frame, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J135" s="9" t="inlineStr">
@@ -9101,7 +9101,7 @@
       </c>
       <c r="I136" s="7" t="inlineStr">
         <is>
-          <t>an off-white cotton kurta with slate grey trousers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an off-white cotton kurta with slate grey trousers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J136" s="7" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="I137" s="9" t="inlineStr">
         <is>
-          <t>a mustard yellow kurta with green embroidered borders displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a mustard yellow kurta with green embroidered borders displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J137" s="9" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="I138" s="7" t="inlineStr">
         <is>
-          <t>a navy hoodie with orange trim and loose joggers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a navy hoodie with orange trim and loose joggers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J138" s="7" t="inlineStr">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="I139" s="9" t="inlineStr">
         <is>
-          <t>an ivory kurta under a maroon embroidered waistcoat displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an ivory kurta under a maroon embroidered waistcoat displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J139" s="9" t="inlineStr">
@@ -9329,7 +9329,7 @@
       </c>
       <c r="I140" s="7" t="inlineStr">
         <is>
-          <t>a royal blue light rain jacket over dark trousers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a royal blue light rain jacket over dark trousers displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J140" s="7" t="inlineStr">
@@ -9386,7 +9386,7 @@
       </c>
       <c r="I141" s="9" t="inlineStr">
         <is>
-          <t>a pink jacket with tiny yellow embroidered light motifs displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a pink jacket with tiny yellow embroidered light motifs displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J141" s="9" t="inlineStr">
@@ -9443,7 +9443,7 @@
       </c>
       <c r="I142" s="7" t="inlineStr">
         <is>
-          <t>a mint-white linen shirt with teal sash displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a mint-white linen shirt with teal sash displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J142" s="7" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="I143" s="9" t="inlineStr">
         <is>
-          <t>a cream sherwani with antique gold embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a cream sherwani with antique gold embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J143" s="9" t="inlineStr">
@@ -9557,7 +9557,7 @@
       </c>
       <c r="I144" s="7" t="inlineStr">
         <is>
-          <t>a crimson padded parka with charcoal trims displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a crimson padded parka with charcoal trims displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J144" s="7" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="I145" s="9" t="inlineStr">
         <is>
-          <t>a jade green athletic wind jacket with lime panels displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a jade green athletic wind jacket with lime panels displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J145" s="9" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="I146" s="7" t="inlineStr">
         <is>
-          <t>a deep violet kurta with glowing orange mirror-work embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a deep violet kurta with glowing orange mirror-work embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J146" s="7" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="I147" s="9" t="inlineStr">
         <is>
-          <t>a black and gold champion outfit with gold kite emblem embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a black and gold champion outfit with gold kite emblem embroidery displayed on an elegant faceless wooden tailor's mannequin, front view, isolated on transparent background, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J147" s="9" t="inlineStr">
@@ -9785,7 +9785,7 @@
       </c>
       <c r="I148" s="7" t="inlineStr">
         <is>
-          <t>a white crocheted prayer cap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a white crocheted prayer cap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J148" s="7" t="inlineStr">
@@ -9842,7 +9842,7 @@
       </c>
       <c r="I149" s="9" t="inlineStr">
         <is>
-          <t>an orange-red baseball-style cap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an orange-red baseball-style cap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J149" s="9" t="inlineStr">
@@ -9899,7 +9899,7 @@
       </c>
       <c r="I150" s="7" t="inlineStr">
         <is>
-          <t>an orange festival turban with a gold brooch, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an orange festival turban with a gold brooch, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J150" s="7" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="I151" s="9" t="inlineStr">
         <is>
-          <t>a blue cotton sweatband, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a blue cotton sweatband, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J151" s="9" t="inlineStr">
@@ -10013,7 +10013,7 @@
       </c>
       <c r="I152" s="7" t="inlineStr">
         <is>
-          <t>stylish black sunglasses, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>stylish black sunglasses, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J152" s="7" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="I153" s="9" t="inlineStr">
         <is>
-          <t>teal aviator wind goggles with leather strap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>teal aviator wind goggles with leather strap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J153" s="9" t="inlineStr">
@@ -10127,7 +10127,7 @@
       </c>
       <c r="I154" s="7" t="inlineStr">
         <is>
-          <t>a brown leather kite carrying bag, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a brown leather kite carrying bag, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J154" s="7" t="inlineStr">
@@ -10184,7 +10184,7 @@
       </c>
       <c r="I155" s="9" t="inlineStr">
         <is>
-          <t>a long crimson woven scarf, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a long crimson woven scarf, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J155" s="9" t="inlineStr">
@@ -10241,7 +10241,7 @@
       </c>
       <c r="I156" s="7" t="inlineStr">
         <is>
-          <t>a spare yellow paper kite tied with a strap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a spare yellow paper kite tied with a strap, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J156" s="7" t="inlineStr">
@@ -10298,7 +10298,7 @@
       </c>
       <c r="I157" s="9" t="inlineStr">
         <is>
-          <t>a small brown leather belt pouch, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small brown leather belt pouch, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J157" s="9" t="inlineStr">
@@ -10355,7 +10355,7 @@
       </c>
       <c r="I158" s="7" t="inlineStr">
         <is>
-          <t>a green embroidered festival sash, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a green embroidered festival sash, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J158" s="7" t="inlineStr">
@@ -10412,7 +10412,7 @@
       </c>
       <c r="I159" s="9" t="inlineStr">
         <is>
-          <t>a leather holster holding a small wooden spool, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a leather holster holding a small wooden spool, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J159" s="9" t="inlineStr">
@@ -10469,7 +10469,7 @@
       </c>
       <c r="I160" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a joyful raised fist with a cut kite string floating away (the famous 'Bo Kata!' cheer), single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a joyful raised fist with a cut kite string floating away (the famous 'Bo Kata!' cheer), single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J160" s="7" t="inlineStr">
@@ -10526,7 +10526,7 @@
       </c>
       <c r="I161" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a thumbs-up hand, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a thumbs-up hand, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J161" s="9" t="inlineStr">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="I162" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a friendly waving hand, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a friendly waving hand, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J162" s="7" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="I163" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a small dancing figure silhouette with motion swirls, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a small dancing figure silhouette with motion swirls, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J163" s="9" t="inlineStr">
@@ -10697,7 +10697,7 @@
       </c>
       <c r="I164" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with two clapping hands with sparkle lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with two clapping hands with sparkle lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J164" s="7" t="inlineStr">
@@ -10754,7 +10754,7 @@
       </c>
       <c r="I165" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a figure bowing respectfully, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a figure bowing respectfully, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J165" s="9" t="inlineStr">
@@ -10811,7 +10811,7 @@
       </c>
       <c r="I166" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a figure spinning with circular motion lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a figure spinning with circular motion lines, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J166" s="7" t="inlineStr">
@@ -10868,7 +10868,7 @@
       </c>
       <c r="I167" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a laughing face with closed happy eyes, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a laughing face with closed happy eyes, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J167" s="9" t="inlineStr">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="I168" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a shrugging figure, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a shrugging figure, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J168" s="7" t="inlineStr">
@@ -10982,7 +10982,7 @@
       </c>
       <c r="I169" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a festive double-headed dhol drum with sticks, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a festive double-headed dhol drum with sticks, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J169" s="9" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="I170" s="7" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a hand saluting, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a hand saluting, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J170" s="7" t="inlineStr">
@@ -11096,7 +11096,7 @@
       </c>
       <c r="I171" s="9" t="inlineStr">
         <is>
-          <t>a round ornate medallion with a hand on a forehead in a facepalm, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round ornate medallion with a hand on a forehead in a facepalm, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J171" s="9" t="inlineStr">
@@ -11153,7 +11153,7 @@
       </c>
       <c r="I172" s="7" t="inlineStr">
         <is>
-          <t>dense old walled city rooftops with brick houses, carved wooden balconies, water tanks and laundry lines, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>dense old walled city rooftops with brick houses, carved wooden balconies, water tanks and laundry lines, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J172" s="7" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="I173" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of dense old walled city rooftops with brick houses, carved wooden balconies, water tanks and laundry lines, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of dense old walled city rooftops with brick houses, carved wooden balconies, water tanks and laundry lines, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J173" s="9" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="I174" s="7" t="inlineStr">
         <is>
-          <t>white and teal houses on cliffs above a sparkling sea, lighthouse in the distance, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>white and teal houses on cliffs above a sparkling sea, lighthouse in the distance, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J174" s="7" t="inlineStr">
@@ -11324,7 +11324,7 @@
       </c>
       <c r="I175" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of white and teal houses on cliffs above a sparkling sea, lighthouse in the distance, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of white and teal houses on cliffs above a sparkling sea, lighthouse in the distance, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J175" s="9" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="I176" s="7" t="inlineStr">
         <is>
-          <t>riverside houses with festival lanterns, boats and stone ghats, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>riverside houses with festival lanterns, boats and stone ghats, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J176" s="7" t="inlineStr">
@@ -11438,7 +11438,7 @@
       </c>
       <c r="I177" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of riverside houses with festival lanterns, boats and stone ghats, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of riverside houses with festival lanterns, boats and stone ghats, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J177" s="9" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="I178" s="7" t="inlineStr">
         <is>
-          <t>a vast palace ground with domed pavilions and manicured gardens, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a vast palace ground with domed pavilions and manicured gardens, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J178" s="7" t="inlineStr">
@@ -11552,7 +11552,7 @@
       </c>
       <c r="I179" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of a vast palace ground with domed pavilions and manicured gardens, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of a vast palace ground with domed pavilions and manicured gardens, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J179" s="9" t="inlineStr">
@@ -11609,7 +11609,7 @@
       </c>
       <c r="I180" s="7" t="inlineStr">
         <is>
-          <t>a terraced village in a green valley with snowy peaks behind, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a terraced village in a green valley with snowy peaks behind, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J180" s="7" t="inlineStr">
@@ -11666,7 +11666,7 @@
       </c>
       <c r="I181" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of a terraced village in a green valley with snowy peaks behind, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of a terraced village in a green valley with snowy peaks behind, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J181" s="9" t="inlineStr">
@@ -11723,7 +11723,7 @@
       </c>
       <c r="I182" s="7" t="inlineStr">
         <is>
-          <t>small rocky islands with stilt houses under dramatic dark storm clouds and shafts of light, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>small rocky islands with stilt houses under dramatic dark storm clouds and shafts of light, kites flying overhead, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J182" s="7" t="inlineStr">
@@ -11780,7 +11780,7 @@
       </c>
       <c r="I183" s="9" t="inlineStr">
         <is>
-          <t>Top-down illustrated antique map of small rocky islands with stilt houses under dramatic dark storm clouds and shafts of light, painted like an old manuscript city plan, soft colours, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Top-down illustrated antique map of small rocky islands with stilt houses under dramatic dark storm clouds and shafts of light, painted like an old manuscript city plan, soft colours, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J183" s="9" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="I184" s="7" t="inlineStr">
         <is>
-          <t>two kites crossing strings one-on-one, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>two kites crossing strings one-on-one, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J184" s="7" t="inlineStr">
@@ -11894,7 +11894,7 @@
       </c>
       <c r="I185" s="9" t="inlineStr">
         <is>
-          <t>two kites duelling with a golden laurel wreath behind, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>two kites duelling with a golden laurel wreath behind, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J185" s="9" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="I186" s="7" t="inlineStr">
         <is>
-          <t>eight colourful kites tangling in a crowded sky, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>eight colourful kites tangling in a crowded sky, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J186" s="7" t="inlineStr">
@@ -12008,7 +12008,7 @@
       </c>
       <c r="I187" s="9" t="inlineStr">
         <is>
-          <t>a carved wooden door slightly open to a rooftop with kites, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a carved wooden door slightly open to a rooftop with kites, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J187" s="9" t="inlineStr">
@@ -12065,7 +12065,7 @@
       </c>
       <c r="I188" s="7" t="inlineStr">
         <is>
-          <t>two groups of kites, saffron team and indigo team, facing each other, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>two groups of kites, saffron team and indigo team, facing each other, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J188" s="7" t="inlineStr">
@@ -12122,7 +12122,7 @@
       </c>
       <c r="I189" s="9" t="inlineStr">
         <is>
-          <t>one proud kite remaining high above many falling kites, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>one proud kite remaining high above many falling kites, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J189" s="9" t="inlineStr">
@@ -12179,7 +12179,7 @@
       </c>
       <c r="I190" s="7" t="inlineStr">
         <is>
-          <t>a kite tied to a practice pole on a quiet rooftop with a friendly helper, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a kite tied to a practice pole on a quiet rooftop with a friendly helper, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J190" s="7" t="inlineStr">
@@ -12236,7 +12236,7 @@
       </c>
       <c r="I191" s="9" t="inlineStr">
         <is>
-          <t>an elder teaching a child to fly a kite on a rooftop, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an elder teaching a child to fly a kite on a rooftop, cinematic wide composition, layered depth, soft atmospheric haze, festival sky full of colourful paper kites, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J191" s="9" t="inlineStr">
@@ -12635,7 +12635,7 @@
       </c>
       <c r="I198" s="7" t="inlineStr">
         <is>
-          <t>a small painted icon of a wooden plank bridge between rooftops, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small painted icon of a wooden plank bridge between rooftops, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J198" s="7" t="inlineStr">
@@ -12692,7 +12692,7 @@
       </c>
       <c r="I199" s="9" t="inlineStr">
         <is>
-          <t>a small painted icon of a swaying rope bridge, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small painted icon of a swaying rope bridge, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J199" s="9" t="inlineStr">
@@ -12749,7 +12749,7 @@
       </c>
       <c r="I200" s="7" t="inlineStr">
         <is>
-          <t>a small painted icon of a wooden ladder, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small painted icon of a wooden ladder, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J200" s="7" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="I201" s="9" t="inlineStr">
         <is>
-          <t>a small painted icon of stone stairs, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small painted icon of stone stairs, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J201" s="9" t="inlineStr">
@@ -12863,7 +12863,7 @@
       </c>
       <c r="I202" s="7" t="inlineStr">
         <is>
-          <t>a stack of three antique gold coins with a tiny kite stamped on them, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a stack of three antique gold coins with a tiny kite stamped on them, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J202" s="7" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="I203" s="9" t="inlineStr">
         <is>
-          <t>a cluster of faceted ruby and emerald gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a cluster of faceted ruby and emerald gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J203" s="9" t="inlineStr">
@@ -12977,7 +12977,7 @@
       </c>
       <c r="I204" s="7" t="inlineStr">
         <is>
-          <t>a bundle of bamboo sticks, a paper sheet and a small thread spool tied together, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a bundle of bamboo sticks, a paper sheet and a small thread spool tied together, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J204" s="7" t="inlineStr">
@@ -13034,7 +13034,7 @@
       </c>
       <c r="I205" s="9" t="inlineStr">
         <is>
-          <t>a small velvet pouch of gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small velvet pouch of gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J205" s="9" t="inlineStr">
@@ -13091,7 +13091,7 @@
       </c>
       <c r="I206" s="7" t="inlineStr">
         <is>
-          <t>a larger cloth bag overflowing with gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a larger cloth bag overflowing with gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J206" s="7" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="I207" s="9" t="inlineStr">
         <is>
-          <t>an ornate wooden treasure chest filled with gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an ornate wooden treasure chest filled with gems, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J207" s="9" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="I208" s="7" t="inlineStr">
         <is>
-          <t>a peaceful clear sky medallion with a single kite and a soft gold ribbon seal, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a peaceful clear sky medallion with a single kite and a soft gold ribbon seal, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J208" s="7" t="inlineStr">
@@ -13262,7 +13262,7 @@
       </c>
       <c r="I209" s="9" t="inlineStr">
         <is>
-          <t>a royal golden scroll pass with an indigo ribbon and a kite seal, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a royal golden scroll pass with an indigo ribbon and a kite seal, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J209" s="9" t="inlineStr">
@@ -13319,7 +13319,7 @@
       </c>
       <c r="I210" s="7" t="inlineStr">
         <is>
-          <t>Wide ornamental festival banner, a spiral of golden kites rising into a twilight sky, gold-leaf arabesque borders top and bottom, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Wide ornamental festival banner, a spiral of golden kites rising into a twilight sky, gold-leaf arabesque borders top and bottom, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J210" s="7" t="inlineStr">
@@ -13376,7 +13376,7 @@
       </c>
       <c r="I211" s="9" t="inlineStr">
         <is>
-          <t>a simple bronze ribbon medallion, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a simple bronze ribbon medallion, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J211" s="9" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="I212" s="7" t="inlineStr">
         <is>
-          <t>a jewelled golden crown medallion, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a jewelled golden crown medallion, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J212" s="7" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="I213" s="9" t="inlineStr">
         <is>
-          <t>a small round gold coin-like level token, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small round gold coin-like level token, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J213" s="9" t="inlineStr">
@@ -13547,7 +13547,7 @@
       </c>
       <c r="I214" s="7" t="inlineStr">
         <is>
-          <t>a wooden crate with a cotton thread ball symbol, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden crate with a cotton thread ball symbol, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J214" s="7" t="inlineStr">
@@ -13604,7 +13604,7 @@
       </c>
       <c r="I215" s="9" t="inlineStr">
         <is>
-          <t>a wooden crate with a spool symbol, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden crate with a spool symbol, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J215" s="9" t="inlineStr">
@@ -13661,7 +13661,7 @@
       </c>
       <c r="I216" s="7" t="inlineStr">
         <is>
-          <t>a small cloth kit with paper patches and glue pot, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a small cloth kit with paper patches and glue pot, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J216" s="7" t="inlineStr">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="I217" s="9" t="inlineStr">
         <is>
-          <t>a crate with fresh thread spools, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a crate with fresh thread spools, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J217" s="9" t="inlineStr">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="I218" s="7" t="inlineStr">
         <is>
-          <t>an ornate carved wooden chest with brass corners and a kite emblem, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>an ornate carved wooden chest with brass corners and a kite emblem, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J218" s="7" t="inlineStr">
@@ -13832,7 +13832,7 @@
       </c>
       <c r="I219" s="9" t="inlineStr">
         <is>
-          <t>the same ornate carved wooden chest open with warm golden light and sparkles rising, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>the same ornate carved wooden chest open with warm golden light and sparkles rising, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J219" s="9" t="inlineStr">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="I220" s="7" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in bronze with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in bronze with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J220" s="7" t="inlineStr">
@@ -13946,7 +13946,7 @@
       </c>
       <c r="I221" s="9" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in polished silver with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in polished silver with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J221" s="9" t="inlineStr">
@@ -14003,7 +14003,7 @@
       </c>
       <c r="I222" s="7" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in rich gold with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in rich gold with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J222" s="7" t="inlineStr">
@@ -14060,7 +14060,7 @@
       </c>
       <c r="I223" s="9" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in pale platinum with pearl with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in pale platinum with pearl with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J223" s="9" t="inlineStr">
@@ -14117,7 +14117,7 @@
       </c>
       <c r="I224" s="7" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in sparkling diamond-blue crystal with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in sparkling diamond-blue crystal with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J224" s="7" t="inlineStr">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="I225" s="9" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in royal purple and gold with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in royal purple and gold with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J225" s="9" t="inlineStr">
@@ -14231,7 +14231,7 @@
       </c>
       <c r="I226" s="7" t="inlineStr">
         <is>
-          <t>a heraldic shield emblem in radiant gold with sun rays and a flying kite crest with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a heraldic shield emblem in radiant gold with sun rays and a flying kite crest with a diamond kite crest and laurel leaves, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J226" s="7" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="I227" s="9" t="inlineStr">
         <is>
-          <t>a kite tail with a ribbon sparkle effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a kite tail with a ribbon sparkle effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J227" s="9" t="inlineStr">
@@ -14345,7 +14345,7 @@
       </c>
       <c r="I228" s="7" t="inlineStr">
         <is>
-          <t>a kite tail with a rainbow trail effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a kite tail with a rainbow trail effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J228" s="7" t="inlineStr">
@@ -14402,7 +14402,7 @@
       </c>
       <c r="I229" s="9" t="inlineStr">
         <is>
-          <t>a kite tail with a firefly tail effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a kite tail with a firefly tail effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J229" s="9" t="inlineStr">
@@ -14459,7 +14459,7 @@
       </c>
       <c r="I230" s="7" t="inlineStr">
         <is>
-          <t>a kite tail with a petal drift effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a kite tail with a petal drift effect, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J230" s="7" t="inlineStr">
@@ -14516,7 +14516,7 @@
       </c>
       <c r="I231" s="9" t="inlineStr">
         <is>
-          <t>a burst of paper confetti in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a burst of paper confetti in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J231" s="9" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="I232" s="7" t="inlineStr">
         <is>
-          <t>a burst of lantern burst in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a burst of lantern burst in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J232" s="7" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="I233" s="9" t="inlineStr">
         <is>
-          <t>a burst of feather swirl in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a burst of feather swirl in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J233" s="9" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="I234" s="7" t="inlineStr">
         <is>
-          <t>a burst of firework in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a burst of firework in the sky, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J234" s="7" t="inlineStr">
@@ -14744,7 +14744,7 @@
       </c>
       <c r="I235" s="9" t="inlineStr">
         <is>
-          <t>a ball of cotton thread in indigo dye colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a ball of cotton thread in indigo dye colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J235" s="9" t="inlineStr">
@@ -14801,7 +14801,7 @@
       </c>
       <c r="I236" s="7" t="inlineStr">
         <is>
-          <t>a ball of cotton thread in rose dye colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a ball of cotton thread in rose dye colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J236" s="7" t="inlineStr">
@@ -14858,7 +14858,7 @@
       </c>
       <c r="I237" s="9" t="inlineStr">
         <is>
-          <t>a ball of cotton thread in gold thread look colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a ball of cotton thread in gold thread look colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J237" s="9" t="inlineStr">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="I238" s="7" t="inlineStr">
         <is>
-          <t>a ball of cotton thread in glow (visual only) colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a ball of cotton thread in glow (visual only) colour, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J238" s="7" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="I239" s="9" t="inlineStr">
         <is>
-          <t>a wooden kite spool decorated with painted wood style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden kite spool decorated with painted wood style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J239" s="9" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="I240" s="7" t="inlineStr">
         <is>
-          <t>a wooden kite spool decorated with brass rim style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden kite spool decorated with brass rim style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J240" s="7" t="inlineStr">
@@ -15086,7 +15086,7 @@
       </c>
       <c r="I241" s="9" t="inlineStr">
         <is>
-          <t>a wooden kite spool decorated with truck art style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden kite spool decorated with truck art style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J241" s="9" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="I242" s="7" t="inlineStr">
         <is>
-          <t>a wooden kite spool decorated with mirror work style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a wooden kite spool decorated with mirror work style ornament, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J242" s="7" t="inlineStr">
@@ -16226,7 +16226,7 @@
       </c>
       <c r="I261" s="9" t="inlineStr">
         <is>
-          <t>a round mission badge with three small kites in a row, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with three small kites in a row, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J261" s="9" t="inlineStr">
@@ -16283,7 +16283,7 @@
       </c>
       <c r="I262" s="7" t="inlineStr">
         <is>
-          <t>a round mission badge with a trophy with two stars, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with a trophy with two stars, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J262" s="7" t="inlineStr">
@@ -16340,7 +16340,7 @@
       </c>
       <c r="I263" s="9" t="inlineStr">
         <is>
-          <t>a round mission badge with five cut thread pieces, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with five cut thread pieces, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J263" s="9" t="inlineStr">
@@ -16397,7 +16397,7 @@
       </c>
       <c r="I264" s="7" t="inlineStr">
         <is>
-          <t>a round mission badge with a crowded sky of kites, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with a crowded sky of kites, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J264" s="7" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="I265" s="9" t="inlineStr">
         <is>
-          <t>a round mission badge with a glowing sweet-spot target, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with a glowing sweet-spot target, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J265" s="9" t="inlineStr">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="I266" s="7" t="inlineStr">
         <is>
-          <t>a round mission badge with an unbroken thread loop, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with an unbroken thread loop, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J266" s="7" t="inlineStr">
@@ -16568,7 +16568,7 @@
       </c>
       <c r="I267" s="9" t="inlineStr">
         <is>
-          <t>a round mission badge with two hands passing a kite, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with two hands passing a kite, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J267" s="9" t="inlineStr">
@@ -16625,7 +16625,7 @@
       </c>
       <c r="I268" s="7" t="inlineStr">
         <is>
-          <t>a round mission badge with crossed kite strings, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a round mission badge with crossed kite strings, single object centred, isolated on a plain transparent background, three-quarter view, soft painted shading, thin antique-gold outline, readable at 64 px, no background scenery, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J268" s="7" t="inlineStr">
@@ -16682,7 +16682,7 @@
       </c>
       <c r="I269" s="9" t="inlineStr">
         <is>
-          <t>a warm rooftop welcome scene with friends waving and kites rising, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a warm rooftop welcome scene with friends waving and kites rising, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J269" s="9" t="inlineStr">
@@ -16739,7 +16739,7 @@
       </c>
       <c r="I270" s="7" t="inlineStr">
         <is>
-          <t>a hand holding a spool and the kite climbing in the sky with motion lines, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>a hand holding a spool and the kite climbing in the sky with motion lines, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J270" s="7" t="inlineStr">
@@ -16796,7 +16796,7 @@
       </c>
       <c r="I271" s="9" t="inlineStr">
         <is>
-          <t>two kites crossing strings with a dramatic spark of friendly competition, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>two kites crossing strings with a dramatic spark of friendly competition, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J271" s="9" t="inlineStr">
@@ -16853,7 +16853,7 @@
       </c>
       <c r="I272" s="7" t="inlineStr">
         <is>
-          <t>players hopping between rooftops on a plank bridge, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>players hopping between rooftops on a plank bridge, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J272" s="7" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="I273" s="9" t="inlineStr">
         <is>
-          <t>four friends on one rooftop celebrating together, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>four friends on one rooftop celebrating together, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J273" s="9" t="inlineStr">
@@ -16967,7 +16967,7 @@
       </c>
       <c r="I274" s="7" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of old weathered red brick wall, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of old weathered red brick wall, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J274" s="7" t="inlineStr">
@@ -17024,7 +17024,7 @@
       </c>
       <c r="I275" s="9" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of lime-washed plaster wall with soft stains, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of lime-washed plaster wall with soft stains, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J275" s="9" t="inlineStr">
@@ -17081,7 +17081,7 @@
       </c>
       <c r="I276" s="7" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of rooftop floor of terracotta tiles, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of rooftop floor of terracotta tiles, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J276" s="7" t="inlineStr">
@@ -17138,7 +17138,7 @@
       </c>
       <c r="I277" s="9" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of carved dark wooden balcony panel (jharokha), flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of carved dark wooden balcony panel (jharokha), flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J277" s="9" t="inlineStr">
@@ -17195,7 +17195,7 @@
       </c>
       <c r="I278" s="7" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of stone jali lattice screen pattern, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of stone jali lattice screen pattern, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J278" s="7" t="inlineStr">
@@ -17252,7 +17252,7 @@
       </c>
       <c r="I279" s="9" t="inlineStr">
         <is>
-          <t>Seamless tileable texture of woven rug pattern, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted South Asian miniature painting style blended with premium mobile game art, gouache and watercolour texture on aged ivory wasli paper, fine gold-leaf filigree accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, masterpiece, highly detailed, original design</t>
+          <t>Seamless tileable texture of woven rug pattern, flat even lighting, top-down orthographic, stylised painterly, game texture, classical hand-painted storybook illustration in a timeless world kite-festival style, premium mobile game art, gouache and watercolour texture on warm ivory paper, fine antique-gold ornament accents, warm golden-hour light, rich jewel tones (saffron, indigo, vermilion, emerald, ivory, antique gold), delicate brushwork, elegant composition, crisp readable silhouette, culturally respectful, welcoming to players worldwide, masterpiece, highly detailed, original design</t>
         </is>
       </c>
       <c r="J279" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Home screen in the owner's glossy design, glossy skins for all screens
Rebuilds the home screen to match docs/design/home_screen_design.jpg: profile
chip with portrait ring and rank, Settings/Inbox, currency bar, icon menu with
chevrons, Daily Missions with progress bars and coin pills, two-column mode
buttons, arena picker with card art, big orange PLAY, loadout bar, and a
behind-the-shoulder home camera. Glossy navy/blue/orange 9-slice skins are
drawn in code (UI/Glossy.cs) and now used by standard UiKit buttons and panels
everywhere; artist sprites (UI kit rows #359+) replace them via Image Mapper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kft94361aqxz3Q9WMshigR
</commit_message>
<xml_diff>
--- a/docs/Kitefall_Image_Assets.xlsx
+++ b/docs/Kitefall_Image_Assets.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image List" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$M$359</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$M$392</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -737,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -775,15 +775,15 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF('Image List'!B2:B359,A2)</f>
+        <f>COUNTIF('Image List'!B2:B392,A2)</f>
         <v/>
       </c>
       <c r="C2">
-        <f>COUNTIFS('Image List'!B2:B359,A2,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A2,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>COUNTIFS('Image List'!B2:B359,A2,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A2,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A2,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A2,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -794,15 +794,15 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Image List'!B2:B359,A3)</f>
+        <f>COUNTIF('Image List'!B2:B392,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS('Image List'!B2:B359,A3,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A3,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>COUNTIFS('Image List'!B2:B359,A3,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A3,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A3,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A3,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -813,15 +813,15 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Image List'!B2:B359,A4)</f>
+        <f>COUNTIF('Image List'!B2:B392,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS('Image List'!B2:B359,A4,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A4,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>COUNTIFS('Image List'!B2:B359,A4,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A4,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A4,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A4,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -832,15 +832,15 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Image List'!B2:B359,A5)</f>
+        <f>COUNTIF('Image List'!B2:B392,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS('Image List'!B2:B359,A5,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A5,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>COUNTIFS('Image List'!B2:B359,A5,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A5,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A5,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A5,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -851,15 +851,15 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Image List'!B2:B359,A6)</f>
+        <f>COUNTIF('Image List'!B2:B392,A6)</f>
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIFS('Image List'!B2:B359,A6,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A6,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>COUNTIFS('Image List'!B2:B359,A6,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A6,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A6,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A6,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -870,15 +870,15 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Image List'!B2:B359,A7)</f>
+        <f>COUNTIF('Image List'!B2:B392,A7)</f>
         <v/>
       </c>
       <c r="C7">
-        <f>COUNTIFS('Image List'!B2:B359,A7,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A7,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>COUNTIFS('Image List'!B2:B359,A7,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A7,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A7,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A7,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -889,15 +889,15 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF('Image List'!B2:B359,A8)</f>
+        <f>COUNTIF('Image List'!B2:B392,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIFS('Image List'!B2:B359,A8,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A8,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>COUNTIFS('Image List'!B2:B359,A8,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A8,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A8,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A8,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -908,15 +908,15 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Image List'!B2:B359,A9)</f>
+        <f>COUNTIF('Image List'!B2:B392,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIFS('Image List'!B2:B359,A9,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A9,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>COUNTIFS('Image List'!B2:B359,A9,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A9,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A9,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A9,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -927,15 +927,15 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIF('Image List'!B2:B359,A10)</f>
+        <f>COUNTIF('Image List'!B2:B392,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIFS('Image List'!B2:B359,A10,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A10,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>COUNTIFS('Image List'!B2:B359,A10,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A10,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A10,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A10,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -946,15 +946,15 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Image List'!B2:B359,A11)</f>
+        <f>COUNTIF('Image List'!B2:B392,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS('Image List'!B2:B359,A11,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A11,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>COUNTIFS('Image List'!B2:B359,A11,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A11,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A11,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A11,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -965,15 +965,15 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Image List'!B2:B359,A12)</f>
+        <f>COUNTIF('Image List'!B2:B392,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS('Image List'!B2:B359,A12,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A12,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>COUNTIFS('Image List'!B2:B359,A12,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A12,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A12,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A12,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -984,15 +984,15 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Image List'!B2:B359,A13)</f>
+        <f>COUNTIF('Image List'!B2:B392,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS('Image List'!B2:B359,A13,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A13,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>COUNTIFS('Image List'!B2:B359,A13,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A13,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A13,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A13,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1003,15 +1003,15 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF('Image List'!B2:B359,A14)</f>
+        <f>COUNTIF('Image List'!B2:B392,A14)</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS('Image List'!B2:B359,A14,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A14,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>COUNTIFS('Image List'!B2:B359,A14,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A14,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A14,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A14,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1022,15 +1022,15 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIF('Image List'!B2:B359,A15)</f>
+        <f>COUNTIF('Image List'!B2:B392,A15)</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS('Image List'!B2:B359,A15,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A15,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>COUNTIFS('Image List'!B2:B359,A15,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A15,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A15,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A15,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1041,15 +1041,15 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIF('Image List'!B2:B359,A16)</f>
+        <f>COUNTIF('Image List'!B2:B392,A16)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS('Image List'!B2:B359,A16,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A16,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>COUNTIFS('Image List'!B2:B359,A16,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A16,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A16,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A16,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1060,15 +1060,15 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF('Image List'!B2:B359,A17)</f>
+        <f>COUNTIF('Image List'!B2:B392,A17)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS('Image List'!B2:B359,A17,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A17,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>COUNTIFS('Image List'!B2:B359,A17,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A17,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A17,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A17,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1079,15 +1079,15 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Image List'!B2:B359,A18)</f>
+        <f>COUNTIF('Image List'!B2:B392,A18)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS('Image List'!B2:B359,A18,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A18,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>COUNTIFS('Image List'!B2:B359,A18,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A18,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A18,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A18,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1098,15 +1098,15 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Image List'!B2:B359,A19)</f>
+        <f>COUNTIF('Image List'!B2:B392,A19)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS('Image List'!B2:B359,A19,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A19,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>COUNTIFS('Image List'!B2:B359,A19,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A19,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A19,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A19,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1117,15 +1117,15 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF('Image List'!B2:B359,A20)</f>
+        <f>COUNTIF('Image List'!B2:B392,A20)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS('Image List'!B2:B359,A20,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A20,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>COUNTIFS('Image List'!B2:B359,A20,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A20,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A20,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A20,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1136,15 +1136,15 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIF('Image List'!B2:B359,A21)</f>
+        <f>COUNTIF('Image List'!B2:B392,A21)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS('Image List'!B2:B359,A21,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A21,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>COUNTIFS('Image List'!B2:B359,A21,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A21,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A21,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A21,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1155,15 +1155,15 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIF('Image List'!B2:B359,A22)</f>
+        <f>COUNTIF('Image List'!B2:B392,A22)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS('Image List'!B2:B359,A22,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A22,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>COUNTIFS('Image List'!B2:B359,A22,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A22,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A22,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A22,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1174,15 +1174,15 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIF('Image List'!B2:B359,A23)</f>
+        <f>COUNTIF('Image List'!B2:B392,A23)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS('Image List'!B2:B359,A23,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A23,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>COUNTIFS('Image List'!B2:B359,A23,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A23,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A23,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A23,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1193,15 +1193,15 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Image List'!B2:B359,A24)</f>
+        <f>COUNTIF('Image List'!B2:B392,A24)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS('Image List'!B2:B359,A24,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A24,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>COUNTIFS('Image List'!B2:B359,A24,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A24,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A24,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A24,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1212,15 +1212,15 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIF('Image List'!B2:B359,A25)</f>
+        <f>COUNTIF('Image List'!B2:B392,A25)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS('Image List'!B2:B359,A25,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A25,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>COUNTIFS('Image List'!B2:B359,A25,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A25,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A25,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A25,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1231,15 +1231,15 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIF('Image List'!B2:B359,A26)</f>
+        <f>COUNTIF('Image List'!B2:B392,A26)</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS('Image List'!B2:B359,A26,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A26,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>COUNTIFS('Image List'!B2:B359,A26,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A26,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A26,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A26,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1250,15 +1250,15 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIF('Image List'!B2:B359,A27)</f>
+        <f>COUNTIF('Image List'!B2:B392,A27)</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS('Image List'!B2:B359,A27,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A27,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>COUNTIFS('Image List'!B2:B359,A27,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A27,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A27,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A27,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1269,15 +1269,15 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIF('Image List'!B2:B359,A28)</f>
+        <f>COUNTIF('Image List'!B2:B392,A28)</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS('Image List'!B2:B359,A28,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A28,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>COUNTIFS('Image List'!B2:B359,A28,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A28,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A28,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A28,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1288,15 +1288,15 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIF('Image List'!B2:B359,A29)</f>
+        <f>COUNTIF('Image List'!B2:B392,A29)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS('Image List'!B2:B359,A29,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A29,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>COUNTIFS('Image List'!B2:B359,A29,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A29,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A29,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A29,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1307,15 +1307,15 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIF('Image List'!B2:B359,A30)</f>
+        <f>COUNTIF('Image List'!B2:B392,A30)</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS('Image List'!B2:B359,A30,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A30,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>COUNTIFS('Image List'!B2:B359,A30,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A30,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A30,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A30,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1326,15 +1326,15 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIF('Image List'!B2:B359,A31)</f>
+        <f>COUNTIF('Image List'!B2:B392,A31)</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS('Image List'!B2:B359,A31,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A31,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>COUNTIFS('Image List'!B2:B359,A31,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A31,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A31,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A31,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1345,15 +1345,15 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIF('Image List'!B2:B359,A32)</f>
+        <f>COUNTIF('Image List'!B2:B392,A32)</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS('Image List'!B2:B359,A32,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A32,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>COUNTIFS('Image List'!B2:B359,A32,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A32,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A32,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A32,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1364,15 +1364,15 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIF('Image List'!B2:B359,A33)</f>
+        <f>COUNTIF('Image List'!B2:B392,A33)</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS('Image List'!B2:B359,A33,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A33,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>COUNTIFS('Image List'!B2:B359,A33,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A33,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A33,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A33,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1383,15 +1383,15 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIF('Image List'!B2:B359,A34)</f>
+        <f>COUNTIF('Image List'!B2:B392,A34)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS('Image List'!B2:B359,A34,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A34,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>COUNTIFS('Image List'!B2:B359,A34,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A34,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A34,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A34,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1402,15 +1402,15 @@
         </is>
       </c>
       <c r="B35">
-        <f>COUNTIF('Image List'!B2:B359,A35)</f>
+        <f>COUNTIF('Image List'!B2:B392,A35)</f>
         <v/>
       </c>
       <c r="C35">
-        <f>COUNTIFS('Image List'!B2:B359,A35,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A35,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>COUNTIFS('Image List'!B2:B359,A35,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A35,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A35,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A35,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1421,15 +1421,15 @@
         </is>
       </c>
       <c r="B36">
-        <f>COUNTIF('Image List'!B2:B359,A36)</f>
+        <f>COUNTIF('Image List'!B2:B392,A36)</f>
         <v/>
       </c>
       <c r="C36">
-        <f>COUNTIFS('Image List'!B2:B359,A36,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A36,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>COUNTIFS('Image List'!B2:B359,A36,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A36,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A36,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A36,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1440,34 +1440,53 @@
         </is>
       </c>
       <c r="B37">
-        <f>COUNTIF('Image List'!B2:B359,A37)</f>
+        <f>COUNTIF('Image List'!B2:B392,A37)</f>
         <v/>
       </c>
       <c r="C37">
-        <f>COUNTIFS('Image List'!B2:B359,A37,'Image List'!G2:G359,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A37,'Image List'!G2:G392,"Critical")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>COUNTIFS('Image List'!B2:B359,A37,'Image List'!K2:K359,"Approved")+COUNTIFS('Image List'!B2:B359,A37,'Image List'!K2:K359,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B392,A37,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A37,'Image List'!K2:K392,"In Unity")</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>COUNTIF('Image List'!B2:B392,A38)</f>
+        <v/>
+      </c>
+      <c r="C38">
+        <f>COUNTIFS('Image List'!B2:B392,A38,'Image List'!G2:G392,"Critical")</f>
+        <v/>
+      </c>
+      <c r="D38">
+        <f>COUNTIFS('Image List'!B2:B392,A38,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A38,'Image List'!K2:K392,"In Unity")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B38" s="5">
-        <f>SUM(B2:B37)</f>
+      <c r="B39" s="5">
+        <f>SUM(B2:B38)</f>
         <v/>
       </c>
-      <c r="C38" s="5">
-        <f>SUM(C2:C37)</f>
+      <c r="C39" s="5">
+        <f>SUM(C2:C38)</f>
         <v/>
       </c>
-      <c r="D38" s="5">
-        <f>SUM(D2:D37)</f>
+      <c r="D39" s="5">
+        <f>SUM(D2:D38)</f>
         <v/>
       </c>
     </row>
@@ -1482,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M359"/>
+  <dimension ref="A1:M392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -21973,10 +21992,1891 @@
       <c r="L359" s="9" t="inlineStr"/>
       <c r="M359" s="9" t="inlineStr"/>
     </row>
+    <row r="360" ht="120" customHeight="1">
+      <c r="A360" s="7" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C360" s="7" t="inlineStr">
+        <is>
+          <t>ui_panel.png</t>
+        </is>
+      </c>
+      <c r="D360" s="7" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E360" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F360" s="7" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G360" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H360" s="7" t="inlineStr">
+        <is>
+          <t>Generic panel (missions, profile, currencies). MUST be 9-slice friendly: plain middle, all detail in the corners/edges. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I360" s="7" t="inlineStr">
+        <is>
+          <t>an empty rounded rectangle panel of deep navy glass with a thin bright blue rim and soft top highlight, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J360" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K360" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L360" s="7" t="inlineStr"/>
+      <c r="M360" s="7" t="inlineStr"/>
+    </row>
+    <row r="361" ht="120" customHeight="1">
+      <c r="A361" s="9" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C361" s="9" t="inlineStr">
+        <is>
+          <t>ui_button_blue.png</t>
+        </is>
+      </c>
+      <c r="D361" s="9" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E361" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F361" s="9" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G361" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H361" s="9" t="inlineStr">
+        <is>
+          <t>Menu buttons (Wardrobe, Squad…). 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I361" s="9" t="inlineStr">
+        <is>
+          <t>an empty rounded rectangle button, navy-to-royal-blue gradient, bright blue rim, glossy top highlight, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J361" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K361" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L361" s="9" t="inlineStr"/>
+      <c r="M361" s="9" t="inlineStr"/>
+    </row>
+    <row r="362" ht="120" customHeight="1">
+      <c r="A362" s="7" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C362" s="7" t="inlineStr">
+        <is>
+          <t>ui_button_selected.png</t>
+        </is>
+      </c>
+      <c r="D362" s="7" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E362" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F362" s="7" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G362" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H362" s="7" t="inlineStr">
+        <is>
+          <t>Selected mode button. 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I362" s="7" t="inlineStr">
+        <is>
+          <t>an empty rounded rectangle button, bright electric blue gradient, white-blue glowing rim, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J362" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K362" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L362" s="7" t="inlineStr"/>
+      <c r="M362" s="7" t="inlineStr"/>
+    </row>
+    <row r="363" ht="120" customHeight="1">
+      <c r="A363" s="9" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C363" s="9" t="inlineStr">
+        <is>
+          <t>ui_button_orange.png</t>
+        </is>
+      </c>
+      <c r="D363" s="9" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E363" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F363" s="9" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G363" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H363" s="9" t="inlineStr">
+        <is>
+          <t>PLAY / Open daily chest. 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I363" s="9" t="inlineStr">
+        <is>
+          <t>an empty large rounded rectangle button, golden-yellow to deep orange gradient, warm light rim and glossy highlight, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J363" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K363" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L363" s="9" t="inlineStr"/>
+      <c r="M363" s="9" t="inlineStr"/>
+    </row>
+    <row r="364" ht="120" customHeight="1">
+      <c r="A364" s="7" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C364" s="7" t="inlineStr">
+        <is>
+          <t>ui_button_locked.png</t>
+        </is>
+      </c>
+      <c r="D364" s="7" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E364" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F364" s="7" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G364" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H364" s="7" t="inlineStr">
+        <is>
+          <t>Locked buttons. 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I364" s="7" t="inlineStr">
+        <is>
+          <t>an empty rounded rectangle button, muted slate grey-blue, dim rim, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J364" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K364" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L364" s="7" t="inlineStr"/>
+      <c r="M364" s="7" t="inlineStr"/>
+    </row>
+    <row r="365" ht="120" customHeight="1">
+      <c r="A365" s="9" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C365" s="9" t="inlineStr">
+        <is>
+          <t>ui_button_green.png</t>
+        </is>
+      </c>
+      <c r="D365" s="9" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E365" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F365" s="9" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G365" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H365" s="9" t="inlineStr">
+        <is>
+          <t>Claim / confirm. 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I365" s="9" t="inlineStr">
+        <is>
+          <t>an empty rounded rectangle button, fresh green gradient with light rim, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J365" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K365" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L365" s="9" t="inlineStr"/>
+      <c r="M365" s="9" t="inlineStr"/>
+    </row>
+    <row r="366" ht="120" customHeight="1">
+      <c r="A366" s="7" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C366" s="7" t="inlineStr">
+        <is>
+          <t>ui_pill.png</t>
+        </is>
+      </c>
+      <c r="D366" s="7" t="inlineStr">
+        <is>
+          <t>256x128</t>
+        </is>
+      </c>
+      <c r="E366" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F366" s="7" t="inlineStr">
+        <is>
+          <t>Every screen (replaces the code-drawn glossy skin)</t>
+        </is>
+      </c>
+      <c r="G366" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H366" s="7" t="inlineStr">
+        <is>
+          <t>Reward pills, + buttons, arrows. 9-slice friendly. Keep it EMPTY – no text, no icons.</t>
+        </is>
+      </c>
+      <c r="I366" s="7" t="inlineStr">
+        <is>
+          <t>an empty small capsule pill shape, very dark navy with a thin blue rim, polished mobile game UI element, glossy deep navy glass with a bright sky-blue rim, soft inner glow, subtle gold accents, clean vector-like edges, high-end casual game interface, front view, isolated on transparent background</t>
+        </is>
+      </c>
+      <c r="J366" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, text, icons</t>
+        </is>
+      </c>
+      <c r="K366" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L366" s="7" t="inlineStr"/>
+      <c r="M366" s="7" t="inlineStr"/>
+    </row>
+    <row r="367" ht="120" customHeight="1">
+      <c r="A367" s="9" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C367" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_gear.png</t>
+        </is>
+      </c>
+      <c r="D367" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E367" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F367" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G367" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H367" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I367" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a settings gear, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J367" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K367" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L367" s="9" t="inlineStr"/>
+      <c r="M367" s="9" t="inlineStr"/>
+    </row>
+    <row r="368" ht="120" customHeight="1">
+      <c r="A368" s="7" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C368" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_mail.png</t>
+        </is>
+      </c>
+      <c r="D368" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E368" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F368" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G368" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H368" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I368" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of an envelope, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J368" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K368" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L368" s="7" t="inlineStr"/>
+      <c r="M368" s="7" t="inlineStr"/>
+    </row>
+    <row r="369" ht="120" customHeight="1">
+      <c r="A369" s="9" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C369" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_shirt.png</t>
+        </is>
+      </c>
+      <c r="D369" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E369" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F369" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G369" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H369" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I369" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a t-shirt, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J369" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K369" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L369" s="9" t="inlineStr"/>
+      <c r="M369" s="9" t="inlineStr"/>
+    </row>
+    <row r="370" ht="120" customHeight="1">
+      <c r="A370" s="7" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C370" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_people.png</t>
+        </is>
+      </c>
+      <c r="D370" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E370" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F370" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G370" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H370" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I370" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of two people silhouettes, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J370" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K370" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L370" s="7" t="inlineStr"/>
+      <c r="M370" s="7" t="inlineStr"/>
+    </row>
+    <row r="371" ht="120" customHeight="1">
+      <c r="A371" s="9" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C371" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_target.png</t>
+        </is>
+      </c>
+      <c r="D371" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E371" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F371" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G371" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H371" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I371" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a target with an arrow, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J371" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K371" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L371" s="9" t="inlineStr"/>
+      <c r="M371" s="9" t="inlineStr"/>
+    </row>
+    <row r="372" ht="120" customHeight="1">
+      <c r="A372" s="7" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C372" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_hangar.png</t>
+        </is>
+      </c>
+      <c r="D372" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E372" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F372" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G372" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H372" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I372" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a kite on a small stand, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J372" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K372" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L372" s="7" t="inlineStr"/>
+      <c r="M372" s="7" t="inlineStr"/>
+    </row>
+    <row r="373" ht="120" customHeight="1">
+      <c r="A373" s="9" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C373" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_wrench.png</t>
+        </is>
+      </c>
+      <c r="D373" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E373" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F373" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G373" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H373" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I373" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a wrench, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J373" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K373" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L373" s="9" t="inlineStr"/>
+      <c r="M373" s="9" t="inlineStr"/>
+    </row>
+    <row r="374" ht="120" customHeight="1">
+      <c r="A374" s="7" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C374" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_cart.png</t>
+        </is>
+      </c>
+      <c r="D374" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E374" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F374" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G374" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H374" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I374" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a shopping cart, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J374" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K374" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L374" s="7" t="inlineStr"/>
+      <c r="M374" s="7" t="inlineStr"/>
+    </row>
+    <row r="375" ht="120" customHeight="1">
+      <c r="A375" s="9" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C375" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_star.png</t>
+        </is>
+      </c>
+      <c r="D375" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E375" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F375" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G375" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H375" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I375" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a five-point star, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J375" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K375" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L375" s="9" t="inlineStr"/>
+      <c r="M375" s="9" t="inlineStr"/>
+    </row>
+    <row r="376" ht="120" customHeight="1">
+      <c r="A376" s="7" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C376" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_trophy.png</t>
+        </is>
+      </c>
+      <c r="D376" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E376" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F376" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G376" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H376" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I376" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a trophy cup, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J376" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K376" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L376" s="7" t="inlineStr"/>
+      <c r="M376" s="7" t="inlineStr"/>
+    </row>
+    <row r="377" ht="120" customHeight="1">
+      <c r="A377" s="9" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C377" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_swords.png</t>
+        </is>
+      </c>
+      <c r="D377" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E377" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F377" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G377" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H377" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I377" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of two crossed kite sticks, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J377" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K377" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L377" s="9" t="inlineStr"/>
+      <c r="M377" s="9" t="inlineStr"/>
+    </row>
+    <row r="378" ht="120" customHeight="1">
+      <c r="A378" s="7" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C378" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_crown.png</t>
+        </is>
+      </c>
+      <c r="D378" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E378" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F378" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G378" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H378" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I378" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a crown, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J378" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K378" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L378" s="7" t="inlineStr"/>
+      <c r="M378" s="7" t="inlineStr"/>
+    </row>
+    <row r="379" ht="120" customHeight="1">
+      <c r="A379" s="9" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C379" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_door.png</t>
+        </is>
+      </c>
+      <c r="D379" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E379" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F379" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G379" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H379" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I379" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of an open door, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J379" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K379" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L379" s="9" t="inlineStr"/>
+      <c r="M379" s="9" t="inlineStr"/>
+    </row>
+    <row r="380" ht="120" customHeight="1">
+      <c r="A380" s="7" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C380" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_kite.png</t>
+        </is>
+      </c>
+      <c r="D380" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E380" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F380" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G380" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H380" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I380" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a diamond kite, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J380" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K380" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L380" s="7" t="inlineStr"/>
+      <c r="M380" s="7" t="inlineStr"/>
+    </row>
+    <row r="381" ht="120" customHeight="1">
+      <c r="A381" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C381" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_chest.png</t>
+        </is>
+      </c>
+      <c r="D381" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E381" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F381" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G381" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H381" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I381" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a treasure chest, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J381" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K381" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L381" s="9" t="inlineStr"/>
+      <c r="M381" s="9" t="inlineStr"/>
+    </row>
+    <row r="382" ht="120" customHeight="1">
+      <c r="A382" s="7" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C382" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_lock.png</t>
+        </is>
+      </c>
+      <c r="D382" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E382" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F382" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G382" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H382" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I382" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a padlock, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J382" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K382" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L382" s="7" t="inlineStr"/>
+      <c r="M382" s="7" t="inlineStr"/>
+    </row>
+    <row r="383" ht="120" customHeight="1">
+      <c r="A383" s="9" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C383" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_clock.png</t>
+        </is>
+      </c>
+      <c r="D383" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E383" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F383" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G383" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H383" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I383" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a clock, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J383" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K383" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L383" s="9" t="inlineStr"/>
+      <c r="M383" s="9" t="inlineStr"/>
+    </row>
+    <row r="384" ht="120" customHeight="1">
+      <c r="A384" s="7" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C384" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_pencil.png</t>
+        </is>
+      </c>
+      <c r="D384" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E384" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F384" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G384" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H384" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I384" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a pencil, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J384" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K384" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L384" s="7" t="inlineStr"/>
+      <c r="M384" s="7" t="inlineStr"/>
+    </row>
+    <row r="385" ht="120" customHeight="1">
+      <c r="A385" s="9" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C385" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_coin.png</t>
+        </is>
+      </c>
+      <c r="D385" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E385" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F385" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G385" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H385" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I385" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a gold coin, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J385" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K385" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L385" s="9" t="inlineStr"/>
+      <c r="M385" s="9" t="inlineStr"/>
+    </row>
+    <row r="386" ht="120" customHeight="1">
+      <c r="A386" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C386" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_gem.png</t>
+        </is>
+      </c>
+      <c r="D386" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E386" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F386" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G386" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H386" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I386" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a blue gem, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J386" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K386" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L386" s="7" t="inlineStr"/>
+      <c r="M386" s="7" t="inlineStr"/>
+    </row>
+    <row r="387" ht="120" customHeight="1">
+      <c r="A387" s="9" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C387" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_parts.png</t>
+        </is>
+      </c>
+      <c r="D387" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E387" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F387" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G387" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H387" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I387" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a crafting parts box, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J387" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K387" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L387" s="9" t="inlineStr"/>
+      <c r="M387" s="9" t="inlineStr"/>
+    </row>
+    <row r="388" ht="120" customHeight="1">
+      <c r="A388" s="7" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C388" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_ribbon.png</t>
+        </is>
+      </c>
+      <c r="D388" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E388" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F388" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G388" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H388" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I388" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a curling ribbon, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J388" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K388" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L388" s="7" t="inlineStr"/>
+      <c r="M388" s="7" t="inlineStr"/>
+    </row>
+    <row r="389" ht="120" customHeight="1">
+      <c r="A389" s="9" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C389" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_thread.png</t>
+        </is>
+      </c>
+      <c r="D389" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E389" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F389" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G389" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H389" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I389" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a ball of cotton thread, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J389" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K389" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L389" s="9" t="inlineStr"/>
+      <c r="M389" s="9" t="inlineStr"/>
+    </row>
+    <row r="390" ht="120" customHeight="1">
+      <c r="A390" s="7" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C390" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_spool.png</t>
+        </is>
+      </c>
+      <c r="D390" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E390" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F390" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G390" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H390" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I390" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a wooden spool, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J390" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K390" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L390" s="7" t="inlineStr"/>
+      <c r="M390" s="7" t="inlineStr"/>
+    </row>
+    <row r="391" ht="120" customHeight="1">
+      <c r="A391" s="9" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" s="9" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C391" s="9" t="inlineStr">
+        <is>
+          <t>ui_icon_chevron_right.png</t>
+        </is>
+      </c>
+      <c r="D391" s="9" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E391" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F391" s="9" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G391" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H391" s="9" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I391" s="9" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a right arrow chevron, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J391" s="9" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K391" s="9" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L391" s="9" t="inlineStr"/>
+      <c r="M391" s="9" t="inlineStr"/>
+    </row>
+    <row r="392" ht="120" customHeight="1">
+      <c r="A392" s="7" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" s="7" t="inlineStr">
+        <is>
+          <t>UI kit</t>
+        </is>
+      </c>
+      <c r="C392" s="7" t="inlineStr">
+        <is>
+          <t>ui_icon_chevron_left.png</t>
+        </is>
+      </c>
+      <c r="D392" s="7" t="inlineStr">
+        <is>
+          <t>128x128</t>
+        </is>
+      </c>
+      <c r="E392" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F392" s="7" t="inlineStr">
+        <is>
+          <t>Home screen + menus icon</t>
+        </is>
+      </c>
+      <c r="G392" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H392" s="7" t="inlineStr">
+        <is>
+          <t>WHITE glyph on transparent background (the game tints it). Bold, simple, readable at 32 px.</t>
+        </is>
+      </c>
+      <c r="I392" s="7" t="inlineStr">
+        <is>
+          <t>a simple flat white silhouette icon of a left arrow chevron, pure white on transparent background, clean bold edges, no shading, game UI glyph</t>
+        </is>
+      </c>
+      <c r="J392" s="7" t="inlineStr">
+        <is>
+          <t>text, letters, numbers, watermark, logo, brand name, signature, frame text, blurry, low resolution, jpeg artifacts, photograph, plastic 3D render, oversaturated neon, extra fingers, deformed hands, distorted face, glass-coated string, metal wire string, nylon string, blades, blood, weapons, real-world flags, copyrighted characters, background scenery, cropped object, multiple objects, drop shadow box, colours, gradients</t>
+        </is>
+      </c>
+      <c r="K392" s="7" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="L392" s="7" t="inlineStr"/>
+      <c r="M392" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M359"/>
+  <autoFilter ref="A1:M392"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K359" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,In progress,Review,Approved,In Unity"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Home screen made from the owner's design picture, with animation
Cuts the owner's design (docs/design/home_screen_design.jpg) into a game kit
(Tools/ArtList/make_home_kit.py): background with the UI and kite removed,
a separate kite sprite, 9-slice button/panel skins and white icons. The home
screen shows the painted picture by default (Settings > Home scene) and
HomeAnimator brings it to life: swaying kite on a line from the flyer's
hand, drifting clouds, birds, sea sparkles and sun glow. UI motion: staggered
slide-ins, PLAY breathing and shine sweep, press bounce on glossy buttons,
coin count-up and mission bar fills. Image list gains the home kit rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kft94361aqxz3Q9WMshigR
</commit_message>
<xml_diff>
--- a/docs/Kitefall_Image_Assets.xlsx
+++ b/docs/Kitefall_Image_Assets.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Image List" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$M$392</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Image List'!$A$1:$M$395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,7 +47,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,6 +146,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -737,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -775,15 +783,15 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF('Image List'!B2:B392,A2)</f>
+        <f>COUNTIF('Image List'!B2:B395,A2)</f>
         <v/>
       </c>
       <c r="C2">
-        <f>COUNTIFS('Image List'!B2:B392,A2,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A2,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D2">
-        <f>COUNTIFS('Image List'!B2:B392,A2,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A2,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A2,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A2,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -794,15 +802,15 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Image List'!B2:B392,A3)</f>
+        <f>COUNTIF('Image List'!B2:B395,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS('Image List'!B2:B392,A3,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A3,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D3">
-        <f>COUNTIFS('Image List'!B2:B392,A3,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A3,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A3,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A3,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -813,15 +821,15 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Image List'!B2:B392,A4)</f>
+        <f>COUNTIF('Image List'!B2:B395,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS('Image List'!B2:B392,A4,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A4,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D4">
-        <f>COUNTIFS('Image List'!B2:B392,A4,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A4,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A4,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A4,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -832,15 +840,15 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF('Image List'!B2:B392,A5)</f>
+        <f>COUNTIF('Image List'!B2:B395,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS('Image List'!B2:B392,A5,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A5,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D5">
-        <f>COUNTIFS('Image List'!B2:B392,A5,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A5,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A5,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A5,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -851,15 +859,15 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Image List'!B2:B392,A6)</f>
+        <f>COUNTIF('Image List'!B2:B395,A6)</f>
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIFS('Image List'!B2:B392,A6,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A6,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>COUNTIFS('Image List'!B2:B392,A6,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A6,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A6,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A6,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -870,15 +878,15 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Image List'!B2:B392,A7)</f>
+        <f>COUNTIF('Image List'!B2:B395,A7)</f>
         <v/>
       </c>
       <c r="C7">
-        <f>COUNTIFS('Image List'!B2:B392,A7,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A7,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D7">
-        <f>COUNTIFS('Image List'!B2:B392,A7,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A7,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A7,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A7,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -889,15 +897,15 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF('Image List'!B2:B392,A8)</f>
+        <f>COUNTIF('Image List'!B2:B395,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIFS('Image List'!B2:B392,A8,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A8,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D8">
-        <f>COUNTIFS('Image List'!B2:B392,A8,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A8,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A8,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A8,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -908,15 +916,15 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Image List'!B2:B392,A9)</f>
+        <f>COUNTIF('Image List'!B2:B395,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIFS('Image List'!B2:B392,A9,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A9,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D9">
-        <f>COUNTIFS('Image List'!B2:B392,A9,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A9,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A9,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A9,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -927,15 +935,15 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIF('Image List'!B2:B392,A10)</f>
+        <f>COUNTIF('Image List'!B2:B395,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIFS('Image List'!B2:B392,A10,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A10,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D10">
-        <f>COUNTIFS('Image List'!B2:B392,A10,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A10,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A10,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A10,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -946,15 +954,15 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIF('Image List'!B2:B392,A11)</f>
+        <f>COUNTIF('Image List'!B2:B395,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS('Image List'!B2:B392,A11,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A11,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D11">
-        <f>COUNTIFS('Image List'!B2:B392,A11,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A11,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A11,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A11,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -965,15 +973,15 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIF('Image List'!B2:B392,A12)</f>
+        <f>COUNTIF('Image List'!B2:B395,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS('Image List'!B2:B392,A12,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A12,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>COUNTIFS('Image List'!B2:B392,A12,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A12,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A12,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A12,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -984,15 +992,15 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIF('Image List'!B2:B392,A13)</f>
+        <f>COUNTIF('Image List'!B2:B395,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS('Image List'!B2:B392,A13,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A13,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D13">
-        <f>COUNTIFS('Image List'!B2:B392,A13,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A13,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A13,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A13,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1003,15 +1011,15 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIF('Image List'!B2:B392,A14)</f>
+        <f>COUNTIF('Image List'!B2:B395,A14)</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS('Image List'!B2:B392,A14,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A14,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D14">
-        <f>COUNTIFS('Image List'!B2:B392,A14,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A14,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A14,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A14,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1022,15 +1030,15 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIF('Image List'!B2:B392,A15)</f>
+        <f>COUNTIF('Image List'!B2:B395,A15)</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS('Image List'!B2:B392,A15,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A15,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D15">
-        <f>COUNTIFS('Image List'!B2:B392,A15,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A15,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A15,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A15,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1041,15 +1049,15 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIF('Image List'!B2:B392,A16)</f>
+        <f>COUNTIF('Image List'!B2:B395,A16)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS('Image List'!B2:B392,A16,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A16,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D16">
-        <f>COUNTIFS('Image List'!B2:B392,A16,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A16,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A16,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A16,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1060,15 +1068,15 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIF('Image List'!B2:B392,A17)</f>
+        <f>COUNTIF('Image List'!B2:B395,A17)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS('Image List'!B2:B392,A17,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A17,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D17">
-        <f>COUNTIFS('Image List'!B2:B392,A17,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A17,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A17,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A17,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1079,15 +1087,15 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIF('Image List'!B2:B392,A18)</f>
+        <f>COUNTIF('Image List'!B2:B395,A18)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS('Image List'!B2:B392,A18,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A18,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D18">
-        <f>COUNTIFS('Image List'!B2:B392,A18,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A18,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A18,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A18,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1098,15 +1106,15 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIF('Image List'!B2:B392,A19)</f>
+        <f>COUNTIF('Image List'!B2:B395,A19)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS('Image List'!B2:B392,A19,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A19,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D19">
-        <f>COUNTIFS('Image List'!B2:B392,A19,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A19,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A19,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A19,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1117,15 +1125,15 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIF('Image List'!B2:B392,A20)</f>
+        <f>COUNTIF('Image List'!B2:B395,A20)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS('Image List'!B2:B392,A20,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A20,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D20">
-        <f>COUNTIFS('Image List'!B2:B392,A20,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A20,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A20,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A20,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1136,15 +1144,15 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIF('Image List'!B2:B392,A21)</f>
+        <f>COUNTIF('Image List'!B2:B395,A21)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS('Image List'!B2:B392,A21,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A21,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D21">
-        <f>COUNTIFS('Image List'!B2:B392,A21,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A21,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A21,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A21,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1155,15 +1163,15 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIF('Image List'!B2:B392,A22)</f>
+        <f>COUNTIF('Image List'!B2:B395,A22)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS('Image List'!B2:B392,A22,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A22,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D22">
-        <f>COUNTIFS('Image List'!B2:B392,A22,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A22,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A22,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A22,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1174,15 +1182,15 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIF('Image List'!B2:B392,A23)</f>
+        <f>COUNTIF('Image List'!B2:B395,A23)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS('Image List'!B2:B392,A23,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A23,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>COUNTIFS('Image List'!B2:B392,A23,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A23,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A23,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A23,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1193,15 +1201,15 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIF('Image List'!B2:B392,A24)</f>
+        <f>COUNTIF('Image List'!B2:B395,A24)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS('Image List'!B2:B392,A24,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A24,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>COUNTIFS('Image List'!B2:B392,A24,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A24,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A24,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A24,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1212,15 +1220,15 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIF('Image List'!B2:B392,A25)</f>
+        <f>COUNTIF('Image List'!B2:B395,A25)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS('Image List'!B2:B392,A25,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A25,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>COUNTIFS('Image List'!B2:B392,A25,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A25,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A25,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A25,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1231,15 +1239,15 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIF('Image List'!B2:B392,A26)</f>
+        <f>COUNTIF('Image List'!B2:B395,A26)</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS('Image List'!B2:B392,A26,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A26,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D26">
-        <f>COUNTIFS('Image List'!B2:B392,A26,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A26,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A26,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A26,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1250,15 +1258,15 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIF('Image List'!B2:B392,A27)</f>
+        <f>COUNTIF('Image List'!B2:B395,A27)</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS('Image List'!B2:B392,A27,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A27,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>COUNTIFS('Image List'!B2:B392,A27,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A27,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A27,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A27,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1269,15 +1277,15 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIF('Image List'!B2:B392,A28)</f>
+        <f>COUNTIF('Image List'!B2:B395,A28)</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS('Image List'!B2:B392,A28,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A28,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D28">
-        <f>COUNTIFS('Image List'!B2:B392,A28,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A28,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A28,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A28,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1288,15 +1296,15 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIF('Image List'!B2:B392,A29)</f>
+        <f>COUNTIF('Image List'!B2:B395,A29)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS('Image List'!B2:B392,A29,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A29,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D29">
-        <f>COUNTIFS('Image List'!B2:B392,A29,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A29,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A29,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A29,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1307,15 +1315,15 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIF('Image List'!B2:B392,A30)</f>
+        <f>COUNTIF('Image List'!B2:B395,A30)</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS('Image List'!B2:B392,A30,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A30,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D30">
-        <f>COUNTIFS('Image List'!B2:B392,A30,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A30,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A30,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A30,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1326,15 +1334,15 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIF('Image List'!B2:B392,A31)</f>
+        <f>COUNTIF('Image List'!B2:B395,A31)</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS('Image List'!B2:B392,A31,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A31,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D31">
-        <f>COUNTIFS('Image List'!B2:B392,A31,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A31,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A31,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A31,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1345,15 +1353,15 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIF('Image List'!B2:B392,A32)</f>
+        <f>COUNTIF('Image List'!B2:B395,A32)</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS('Image List'!B2:B392,A32,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A32,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D32">
-        <f>COUNTIFS('Image List'!B2:B392,A32,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A32,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A32,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A32,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1364,15 +1372,15 @@
         </is>
       </c>
       <c r="B33">
-        <f>COUNTIF('Image List'!B2:B392,A33)</f>
+        <f>COUNTIF('Image List'!B2:B395,A33)</f>
         <v/>
       </c>
       <c r="C33">
-        <f>COUNTIFS('Image List'!B2:B392,A33,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A33,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D33">
-        <f>COUNTIFS('Image List'!B2:B392,A33,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A33,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A33,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A33,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1383,15 +1391,15 @@
         </is>
       </c>
       <c r="B34">
-        <f>COUNTIF('Image List'!B2:B392,A34)</f>
+        <f>COUNTIF('Image List'!B2:B395,A34)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>COUNTIFS('Image List'!B2:B392,A34,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A34,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D34">
-        <f>COUNTIFS('Image List'!B2:B392,A34,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A34,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A34,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A34,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1402,15 +1410,15 @@
         </is>
       </c>
       <c r="B35">
-        <f>COUNTIF('Image List'!B2:B392,A35)</f>
+        <f>COUNTIF('Image List'!B2:B395,A35)</f>
         <v/>
       </c>
       <c r="C35">
-        <f>COUNTIFS('Image List'!B2:B392,A35,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A35,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D35">
-        <f>COUNTIFS('Image List'!B2:B392,A35,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A35,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A35,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A35,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1421,15 +1429,15 @@
         </is>
       </c>
       <c r="B36">
-        <f>COUNTIF('Image List'!B2:B392,A36)</f>
+        <f>COUNTIF('Image List'!B2:B395,A36)</f>
         <v/>
       </c>
       <c r="C36">
-        <f>COUNTIFS('Image List'!B2:B392,A36,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A36,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D36">
-        <f>COUNTIFS('Image List'!B2:B392,A36,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A36,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A36,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A36,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1440,15 +1448,15 @@
         </is>
       </c>
       <c r="B37">
-        <f>COUNTIF('Image List'!B2:B392,A37)</f>
+        <f>COUNTIF('Image List'!B2:B395,A37)</f>
         <v/>
       </c>
       <c r="C37">
-        <f>COUNTIFS('Image List'!B2:B392,A37,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A37,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D37">
-        <f>COUNTIFS('Image List'!B2:B392,A37,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A37,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A37,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A37,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
@@ -1459,34 +1467,53 @@
         </is>
       </c>
       <c r="B38">
-        <f>COUNTIF('Image List'!B2:B392,A38)</f>
+        <f>COUNTIF('Image List'!B2:B395,A38)</f>
         <v/>
       </c>
       <c r="C38">
-        <f>COUNTIFS('Image List'!B2:B392,A38,'Image List'!G2:G392,"Critical")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A38,'Image List'!G2:G395,"Critical")</f>
         <v/>
       </c>
       <c r="D38">
-        <f>COUNTIFS('Image List'!B2:B392,A38,'Image List'!K2:K392,"Approved")+COUNTIFS('Image List'!B2:B392,A38,'Image List'!K2:K392,"In Unity")</f>
+        <f>COUNTIFS('Image List'!B2:B395,A38,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A38,'Image List'!K2:K395,"In Unity")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Home design</t>
+        </is>
+      </c>
+      <c r="B39">
+        <f>COUNTIF('Image List'!B2:B395,A39)</f>
+        <v/>
+      </c>
+      <c r="C39">
+        <f>COUNTIFS('Image List'!B2:B395,A39,'Image List'!G2:G395,"Critical")</f>
+        <v/>
+      </c>
+      <c r="D39">
+        <f>COUNTIFS('Image List'!B2:B395,A39,'Image List'!K2:K395,"Approved")+COUNTIFS('Image List'!B2:B395,A39,'Image List'!K2:K395,"In Unity")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B39" s="5">
-        <f>SUM(B2:B38)</f>
+      <c r="B40" s="5">
+        <f>SUM(B2:B39)</f>
         <v/>
       </c>
-      <c r="C39" s="5">
-        <f>SUM(C2:C38)</f>
+      <c r="C40" s="5">
+        <f>SUM(C2:C39)</f>
         <v/>
       </c>
-      <c r="D39" s="5">
-        <f>SUM(D2:D38)</f>
+      <c r="D40" s="5">
+        <f>SUM(D2:D39)</f>
         <v/>
       </c>
     </row>
@@ -1501,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M392"/>
+  <dimension ref="A1:M395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -23873,10 +23900,169 @@
       <c r="L392" s="7" t="inlineStr"/>
       <c r="M392" s="7" t="inlineStr"/>
     </row>
+    <row r="393" ht="120" customHeight="1">
+      <c r="A393" s="9" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" s="9" t="inlineStr">
+        <is>
+          <t>Home design</t>
+        </is>
+      </c>
+      <c r="C393" s="9" t="inlineStr">
+        <is>
+          <t>home_background.jpg</t>
+        </is>
+      </c>
+      <c r="D393" s="9" t="inlineStr">
+        <is>
+          <t>1920x1080</t>
+        </is>
+      </c>
+      <c r="E393" s="9" t="inlineStr">
+        <is>
+          <t>JPG</t>
+        </is>
+      </c>
+      <c r="F393" s="9" t="inlineStr">
+        <is>
+          <t>Home screen painted background (Settings ▸ Home scene ▸ Painted design)</t>
+        </is>
+      </c>
+      <c r="G393" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H393" s="9" t="inlineStr">
+        <is>
+          <t>ALREADY MADE from docs/design/home_screen_design.jpg (UI removed, kite removed). Replace only if you want a new home picture – keep the flyer at the same spot.</t>
+        </is>
+      </c>
+      <c r="I393" s="9" t="inlineStr">
+        <is>
+          <t>Made from the owner's own design picture – no AI prompt needed.</t>
+        </is>
+      </c>
+      <c r="J393" s="9" t="inlineStr"/>
+      <c r="K393" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L393" s="9" t="inlineStr"/>
+      <c r="M393" s="9" t="inlineStr"/>
+    </row>
+    <row r="394" ht="120" customHeight="1">
+      <c r="A394" s="7" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" s="7" t="inlineStr">
+        <is>
+          <t>Home design</t>
+        </is>
+      </c>
+      <c r="C394" s="7" t="inlineStr">
+        <is>
+          <t>home_kite.png</t>
+        </is>
+      </c>
+      <c r="D394" s="7" t="inlineStr">
+        <is>
+          <t>195x175</t>
+        </is>
+      </c>
+      <c r="E394" s="7" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F394" s="7" t="inlineStr">
+        <is>
+          <t>Animated kite on the home picture</t>
+        </is>
+      </c>
+      <c r="G394" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H394" s="7" t="inlineStr">
+        <is>
+          <t>ALREADY MADE (cut from the design). Kite + tail only, transparent background.</t>
+        </is>
+      </c>
+      <c r="I394" s="7" t="inlineStr">
+        <is>
+          <t>Made from the owner's own design picture – no AI prompt needed.</t>
+        </is>
+      </c>
+      <c r="J394" s="7" t="inlineStr"/>
+      <c r="K394" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L394" s="7" t="inlineStr"/>
+      <c r="M394" s="7" t="inlineStr"/>
+    </row>
+    <row r="395" ht="120" customHeight="1">
+      <c r="A395" s="9" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" s="9" t="inlineStr">
+        <is>
+          <t>Home design</t>
+        </is>
+      </c>
+      <c r="C395" s="9" t="inlineStr">
+        <is>
+          <t>ui_button_play.png</t>
+        </is>
+      </c>
+      <c r="D395" s="9" t="inlineStr">
+        <is>
+          <t>460x128</t>
+        </is>
+      </c>
+      <c r="E395" s="9" t="inlineStr">
+        <is>
+          <t>PNG (transparent)</t>
+        </is>
+      </c>
+      <c r="F395" s="9" t="inlineStr">
+        <is>
+          <t>PLAY button skin (9-slice)</t>
+        </is>
+      </c>
+      <c r="G395" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H395" s="9" t="inlineStr">
+        <is>
+          <t>ALREADY MADE (cut from the design, text removed). Keep it EMPTY.</t>
+        </is>
+      </c>
+      <c r="I395" s="9" t="inlineStr">
+        <is>
+          <t>Made from the owner's own design picture – no AI prompt needed.</t>
+        </is>
+      </c>
+      <c r="J395" s="9" t="inlineStr"/>
+      <c r="K395" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L395" s="9" t="inlineStr"/>
+      <c r="M395" s="9" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M392"/>
+  <autoFilter ref="A1:M395"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K392" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K395" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,In progress,Review,Approved,In Unity"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>